<commit_message>
update Adddatato... run error case outpu
Adjusted the data_plot class such that the output data functions are now able to generate output despite a scdp run resulting in an error.

While outputting, it does now not ruin the file format, making post processing easier.
</commit_message>
<xml_diff>
--- a/code_developments_for_publications/scdp_excel/scdp_comparison.xlsx
+++ b/code_developments_for_publications/scdp_excel/scdp_comparison.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\BSO-toolbox-V2\code_developments_for_publications\scdp_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4E1BD3-D956-44DE-A330-54E18F154C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37D022A-FB98-4F7D-A340-5EF99AAF6365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,86 +17,182 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$AH$3</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$AH$4:$AH$25</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">Sheet1!$CQ$3</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">Sheet1!$CQ$4:$CQ$25</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">Sheet1!$EA$3</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">Sheet1!$EA$4:$EA$25</definedName>
-    <definedName name="_xlchart.v1.14" hidden="1">Sheet1!$U$3</definedName>
-    <definedName name="_xlchart.v1.15" hidden="1">Sheet1!$U$4:$U$25</definedName>
-    <definedName name="_xlchart.v1.16" hidden="1">Sheet1!$AJ$3</definedName>
-    <definedName name="_xlchart.v1.17" hidden="1">Sheet1!$AJ$4:$AJ$25</definedName>
-    <definedName name="_xlchart.v1.18" hidden="1">Sheet1!$BT$3</definedName>
-    <definedName name="_xlchart.v1.19" hidden="1">Sheet1!$BT$4:$BT$25</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$BR$3</definedName>
-    <definedName name="_xlchart.v1.20" hidden="1">Sheet1!$DD$3</definedName>
-    <definedName name="_xlchart.v1.21" hidden="1">Sheet1!$DD$4:$DD$25</definedName>
-    <definedName name="_xlchart.v1.22" hidden="1">Sheet1!$EN$3</definedName>
-    <definedName name="_xlchart.v1.23" hidden="1">Sheet1!$EN$4:$EN$25</definedName>
-    <definedName name="_xlchart.v1.24" hidden="1">Sheet1!$BE$3</definedName>
-    <definedName name="_xlchart.v1.25" hidden="1">Sheet1!$BE$4:$BE$25</definedName>
-    <definedName name="_xlchart.v1.26" hidden="1">Sheet1!$CO$3</definedName>
-    <definedName name="_xlchart.v1.27" hidden="1">Sheet1!$CO$4:$CO$25</definedName>
-    <definedName name="_xlchart.v1.28" hidden="1">Sheet1!$DY$3</definedName>
-    <definedName name="_xlchart.v1.29" hidden="1">Sheet1!$DY$4:$DY$25</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$BR$4:$BR$25</definedName>
-    <definedName name="_xlchart.v1.30" hidden="1">Sheet1!$S$3</definedName>
-    <definedName name="_xlchart.v1.31" hidden="1">Sheet1!$S$4:$S$25</definedName>
-    <definedName name="_xlchart.v1.32" hidden="1">Sheet1!$AI$3</definedName>
-    <definedName name="_xlchart.v1.33" hidden="1">Sheet1!$AI$4:$AI$25</definedName>
-    <definedName name="_xlchart.v1.34" hidden="1">Sheet1!$AJ$3</definedName>
-    <definedName name="_xlchart.v1.35" hidden="1">Sheet1!$AJ$4:$AJ$25</definedName>
-    <definedName name="_xlchart.v1.36" hidden="1">Sheet1!$AU$3</definedName>
-    <definedName name="_xlchart.v1.37" hidden="1">Sheet1!$AU$4:$AU$25</definedName>
-    <definedName name="_xlchart.v1.38" hidden="1">Sheet1!$AV$3</definedName>
-    <definedName name="_xlchart.v1.39" hidden="1">Sheet1!$AV$4:$AV$25</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$DB$3</definedName>
-    <definedName name="_xlchart.v1.40" hidden="1">Sheet1!$BG$3</definedName>
-    <definedName name="_xlchart.v1.41" hidden="1">Sheet1!$BG$4:$BG$25</definedName>
-    <definedName name="_xlchart.v1.42" hidden="1">Sheet1!$BH$3</definedName>
-    <definedName name="_xlchart.v1.43" hidden="1">Sheet1!$BH$4:$BH$25</definedName>
-    <definedName name="_xlchart.v1.44" hidden="1">Sheet1!$BS$3</definedName>
-    <definedName name="_xlchart.v1.45" hidden="1">Sheet1!$BS$4:$BS$25</definedName>
-    <definedName name="_xlchart.v1.46" hidden="1">Sheet1!$BT$3</definedName>
-    <definedName name="_xlchart.v1.47" hidden="1">Sheet1!$BT$4:$BT$25</definedName>
-    <definedName name="_xlchart.v1.48" hidden="1">Sheet1!$CE$3</definedName>
-    <definedName name="_xlchart.v1.49" hidden="1">Sheet1!$CE$4:$CE$25</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$DB$4:$DB$25</definedName>
-    <definedName name="_xlchart.v1.50" hidden="1">Sheet1!$CF$3</definedName>
-    <definedName name="_xlchart.v1.51" hidden="1">Sheet1!$CF$4:$CF$25</definedName>
-    <definedName name="_xlchart.v1.52" hidden="1">Sheet1!$CQ$3</definedName>
-    <definedName name="_xlchart.v1.53" hidden="1">Sheet1!$CQ$4:$CQ$25</definedName>
-    <definedName name="_xlchart.v1.54" hidden="1">Sheet1!$CR$3</definedName>
-    <definedName name="_xlchart.v1.55" hidden="1">Sheet1!$CR$4:$CR$25</definedName>
-    <definedName name="_xlchart.v1.56" hidden="1">Sheet1!$DC$3</definedName>
-    <definedName name="_xlchart.v1.57" hidden="1">Sheet1!$DC$4:$DC$25</definedName>
-    <definedName name="_xlchart.v1.58" hidden="1">Sheet1!$DD$3</definedName>
-    <definedName name="_xlchart.v1.59" hidden="1">Sheet1!$DD$4:$DD$25</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$EL$3</definedName>
-    <definedName name="_xlchart.v1.60" hidden="1">Sheet1!$DO$3</definedName>
-    <definedName name="_xlchart.v1.61" hidden="1">Sheet1!$DO$4:$DO$25</definedName>
-    <definedName name="_xlchart.v1.62" hidden="1">Sheet1!$DP$3</definedName>
-    <definedName name="_xlchart.v1.63" hidden="1">Sheet1!$DP$4:$DP$25</definedName>
-    <definedName name="_xlchart.v1.64" hidden="1">Sheet1!$EA$3:$EB$3</definedName>
-    <definedName name="_xlchart.v1.65" hidden="1">Sheet1!$EA$4:$EA$25</definedName>
-    <definedName name="_xlchart.v1.66" hidden="1">Sheet1!$EB$3</definedName>
-    <definedName name="_xlchart.v1.67" hidden="1">Sheet1!$EB$4:$EB$25</definedName>
-    <definedName name="_xlchart.v1.68" hidden="1">Sheet1!$EM$3</definedName>
-    <definedName name="_xlchart.v1.69" hidden="1">Sheet1!$EM$4:$EM$25</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$EL$4:$EL$25</definedName>
-    <definedName name="_xlchart.v1.70" hidden="1">Sheet1!$EN$3</definedName>
-    <definedName name="_xlchart.v1.71" hidden="1">Sheet1!$EN$4:$EN$25</definedName>
-    <definedName name="_xlchart.v1.72" hidden="1">Sheet1!$EY$3</definedName>
-    <definedName name="_xlchart.v1.73" hidden="1">Sheet1!$EY$4:$EY$25</definedName>
-    <definedName name="_xlchart.v1.74" hidden="1">Sheet1!$EZ$3</definedName>
-    <definedName name="_xlchart.v1.75" hidden="1">Sheet1!$EZ$4:$EZ$25</definedName>
-    <definedName name="_xlchart.v1.76" hidden="1">Sheet1!$U$3</definedName>
-    <definedName name="_xlchart.v1.77" hidden="1">Sheet1!$U$4:$U$25</definedName>
-    <definedName name="_xlchart.v1.78" hidden="1">Sheet1!$V$3</definedName>
-    <definedName name="_xlchart.v1.79" hidden="1">Sheet1!$V$4:$V$25</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$AI$3</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$AI$4:$AI$25</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Sheet1!$BH$3</definedName>
+    <definedName name="_xlchart.v1.100" hidden="1">Sheet1!$CQ$3</definedName>
+    <definedName name="_xlchart.v1.101" hidden="1">Sheet1!$CQ$4:$CQ$25</definedName>
+    <definedName name="_xlchart.v1.102" hidden="1">Sheet1!$CR$3</definedName>
+    <definedName name="_xlchart.v1.103" hidden="1">Sheet1!$CR$4:$CR$25</definedName>
+    <definedName name="_xlchart.v1.104" hidden="1">Sheet1!$DC$3</definedName>
+    <definedName name="_xlchart.v1.105" hidden="1">Sheet1!$DC$4:$DC$25</definedName>
+    <definedName name="_xlchart.v1.106" hidden="1">Sheet1!$DD$3</definedName>
+    <definedName name="_xlchart.v1.107" hidden="1">Sheet1!$DD$4:$DD$25</definedName>
+    <definedName name="_xlchart.v1.108" hidden="1">Sheet1!$DO$3</definedName>
+    <definedName name="_xlchart.v1.109" hidden="1">Sheet1!$DO$4:$DO$25</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Sheet1!$BH$4:$BH$25</definedName>
+    <definedName name="_xlchart.v1.110" hidden="1">Sheet1!$DP$3</definedName>
+    <definedName name="_xlchart.v1.111" hidden="1">Sheet1!$DP$4:$DP$25</definedName>
+    <definedName name="_xlchart.v1.112" hidden="1">Sheet1!$EA$3:$EB$3</definedName>
+    <definedName name="_xlchart.v1.113" hidden="1">Sheet1!$EA$4:$EA$25</definedName>
+    <definedName name="_xlchart.v1.114" hidden="1">Sheet1!$EB$3</definedName>
+    <definedName name="_xlchart.v1.115" hidden="1">Sheet1!$EB$4:$EB$25</definedName>
+    <definedName name="_xlchart.v1.116" hidden="1">Sheet1!$EM$3</definedName>
+    <definedName name="_xlchart.v1.117" hidden="1">Sheet1!$EM$4:$EM$25</definedName>
+    <definedName name="_xlchart.v1.118" hidden="1">Sheet1!$EN$3</definedName>
+    <definedName name="_xlchart.v1.119" hidden="1">Sheet1!$EN$4:$EN$25</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Sheet1!$BS$3</definedName>
+    <definedName name="_xlchart.v1.120" hidden="1">Sheet1!$EY$3</definedName>
+    <definedName name="_xlchart.v1.121" hidden="1">Sheet1!$EY$4:$EY$25</definedName>
+    <definedName name="_xlchart.v1.122" hidden="1">Sheet1!$EZ$3</definedName>
+    <definedName name="_xlchart.v1.123" hidden="1">Sheet1!$EZ$4:$EZ$25</definedName>
+    <definedName name="_xlchart.v1.124" hidden="1">Sheet1!$U$3</definedName>
+    <definedName name="_xlchart.v1.125" hidden="1">Sheet1!$U$4:$U$25</definedName>
+    <definedName name="_xlchart.v1.126" hidden="1">Sheet1!$V$3</definedName>
+    <definedName name="_xlchart.v1.127" hidden="1">Sheet1!$V$4:$V$25</definedName>
+    <definedName name="_xlchart.v1.128" hidden="1">Sheet1!$AI$3</definedName>
+    <definedName name="_xlchart.v1.129" hidden="1">Sheet1!$AI$4:$AI$25</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Sheet1!$BS$4:$BS$25</definedName>
+    <definedName name="_xlchart.v1.130" hidden="1">Sheet1!$AJ$3</definedName>
+    <definedName name="_xlchart.v1.131" hidden="1">Sheet1!$AJ$4:$AJ$25</definedName>
+    <definedName name="_xlchart.v1.132" hidden="1">Sheet1!$AU$3</definedName>
+    <definedName name="_xlchart.v1.133" hidden="1">Sheet1!$AU$4:$AU$25</definedName>
+    <definedName name="_xlchart.v1.134" hidden="1">Sheet1!$AV$3</definedName>
+    <definedName name="_xlchart.v1.135" hidden="1">Sheet1!$AV$4:$AV$25</definedName>
+    <definedName name="_xlchart.v1.136" hidden="1">Sheet1!$BG$3</definedName>
+    <definedName name="_xlchart.v1.137" hidden="1">Sheet1!$BG$4:$BG$25</definedName>
+    <definedName name="_xlchart.v1.138" hidden="1">Sheet1!$BH$3</definedName>
+    <definedName name="_xlchart.v1.139" hidden="1">Sheet1!$BH$4:$BH$25</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Sheet1!$BT$3</definedName>
+    <definedName name="_xlchart.v1.140" hidden="1">Sheet1!$BS$3</definedName>
+    <definedName name="_xlchart.v1.141" hidden="1">Sheet1!$BS$4:$BS$25</definedName>
+    <definedName name="_xlchart.v1.142" hidden="1">Sheet1!$BT$3</definedName>
+    <definedName name="_xlchart.v1.143" hidden="1">Sheet1!$BT$4:$BT$25</definedName>
+    <definedName name="_xlchart.v1.144" hidden="1">Sheet1!$CE$3</definedName>
+    <definedName name="_xlchart.v1.145" hidden="1">Sheet1!$CE$4:$CE$25</definedName>
+    <definedName name="_xlchart.v1.146" hidden="1">Sheet1!$CF$3</definedName>
+    <definedName name="_xlchart.v1.147" hidden="1">Sheet1!$CF$4:$CF$25</definedName>
+    <definedName name="_xlchart.v1.148" hidden="1">Sheet1!$CQ$3</definedName>
+    <definedName name="_xlchart.v1.149" hidden="1">Sheet1!$CQ$4:$CQ$25</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Sheet1!$BT$4:$BT$25</definedName>
+    <definedName name="_xlchart.v1.150" hidden="1">Sheet1!$CR$3</definedName>
+    <definedName name="_xlchart.v1.151" hidden="1">Sheet1!$CR$4:$CR$25</definedName>
+    <definedName name="_xlchart.v1.152" hidden="1">Sheet1!$DC$3</definedName>
+    <definedName name="_xlchart.v1.153" hidden="1">Sheet1!$DC$4:$DC$25</definedName>
+    <definedName name="_xlchart.v1.154" hidden="1">Sheet1!$DD$3</definedName>
+    <definedName name="_xlchart.v1.155" hidden="1">Sheet1!$DD$4:$DD$25</definedName>
+    <definedName name="_xlchart.v1.156" hidden="1">Sheet1!$DO$3</definedName>
+    <definedName name="_xlchart.v1.157" hidden="1">Sheet1!$DO$4:$DO$25</definedName>
+    <definedName name="_xlchart.v1.158" hidden="1">Sheet1!$DP$3</definedName>
+    <definedName name="_xlchart.v1.159" hidden="1">Sheet1!$DP$4:$DP$25</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">Sheet1!$CE$3</definedName>
+    <definedName name="_xlchart.v1.160" hidden="1">Sheet1!$EA$3:$EB$3</definedName>
+    <definedName name="_xlchart.v1.161" hidden="1">Sheet1!$EA$4:$EA$25</definedName>
+    <definedName name="_xlchart.v1.162" hidden="1">Sheet1!$EB$3</definedName>
+    <definedName name="_xlchart.v1.163" hidden="1">Sheet1!$EB$4:$EB$25</definedName>
+    <definedName name="_xlchart.v1.164" hidden="1">Sheet1!$EM$3</definedName>
+    <definedName name="_xlchart.v1.165" hidden="1">Sheet1!$EM$4:$EM$25</definedName>
+    <definedName name="_xlchart.v1.166" hidden="1">Sheet1!$EN$3</definedName>
+    <definedName name="_xlchart.v1.167" hidden="1">Sheet1!$EN$4:$EN$25</definedName>
+    <definedName name="_xlchart.v1.168" hidden="1">Sheet1!$EY$3</definedName>
+    <definedName name="_xlchart.v1.169" hidden="1">Sheet1!$EY$4:$EY$25</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Sheet1!$CE$4:$CE$25</definedName>
+    <definedName name="_xlchart.v1.170" hidden="1">Sheet1!$EZ$3</definedName>
+    <definedName name="_xlchart.v1.171" hidden="1">Sheet1!$EZ$4:$EZ$25</definedName>
+    <definedName name="_xlchart.v1.172" hidden="1">Sheet1!$U$3</definedName>
+    <definedName name="_xlchart.v1.173" hidden="1">Sheet1!$U$4:$U$25</definedName>
+    <definedName name="_xlchart.v1.174" hidden="1">Sheet1!$V$3</definedName>
+    <definedName name="_xlchart.v1.175" hidden="1">Sheet1!$V$4:$V$25</definedName>
+    <definedName name="_xlchart.v1.18" hidden="1">Sheet1!$CF$3</definedName>
+    <definedName name="_xlchart.v1.19" hidden="1">Sheet1!$CF$4:$CF$25</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$AJ$3</definedName>
+    <definedName name="_xlchart.v1.20" hidden="1">Sheet1!$CQ$3</definedName>
+    <definedName name="_xlchart.v1.21" hidden="1">Sheet1!$CQ$4:$CQ$25</definedName>
+    <definedName name="_xlchart.v1.22" hidden="1">Sheet1!$CR$3</definedName>
+    <definedName name="_xlchart.v1.23" hidden="1">Sheet1!$CR$4:$CR$25</definedName>
+    <definedName name="_xlchart.v1.24" hidden="1">Sheet1!$DC$3</definedName>
+    <definedName name="_xlchart.v1.25" hidden="1">Sheet1!$DC$4:$DC$25</definedName>
+    <definedName name="_xlchart.v1.26" hidden="1">Sheet1!$DD$3</definedName>
+    <definedName name="_xlchart.v1.27" hidden="1">Sheet1!$DD$4:$DD$25</definedName>
+    <definedName name="_xlchart.v1.28" hidden="1">Sheet1!$DO$3</definedName>
+    <definedName name="_xlchart.v1.29" hidden="1">Sheet1!$DO$4:$DO$25</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$AJ$4:$AJ$25</definedName>
+    <definedName name="_xlchart.v1.30" hidden="1">Sheet1!$DP$3</definedName>
+    <definedName name="_xlchart.v1.31" hidden="1">Sheet1!$DP$4:$DP$25</definedName>
+    <definedName name="_xlchart.v1.32" hidden="1">Sheet1!$EA$3:$EB$3</definedName>
+    <definedName name="_xlchart.v1.33" hidden="1">Sheet1!$EA$4:$EA$25</definedName>
+    <definedName name="_xlchart.v1.34" hidden="1">Sheet1!$EB$3</definedName>
+    <definedName name="_xlchart.v1.35" hidden="1">Sheet1!$EB$4:$EB$25</definedName>
+    <definedName name="_xlchart.v1.36" hidden="1">Sheet1!$EM$3</definedName>
+    <definedName name="_xlchart.v1.37" hidden="1">Sheet1!$EM$4:$EM$25</definedName>
+    <definedName name="_xlchart.v1.38" hidden="1">Sheet1!$EN$3</definedName>
+    <definedName name="_xlchart.v1.39" hidden="1">Sheet1!$EN$4:$EN$25</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$AU$3</definedName>
+    <definedName name="_xlchart.v1.40" hidden="1">Sheet1!$EY$3</definedName>
+    <definedName name="_xlchart.v1.41" hidden="1">Sheet1!$EY$4:$EY$25</definedName>
+    <definedName name="_xlchart.v1.42" hidden="1">Sheet1!$EZ$3</definedName>
+    <definedName name="_xlchart.v1.43" hidden="1">Sheet1!$EZ$4:$EZ$25</definedName>
+    <definedName name="_xlchart.v1.44" hidden="1">Sheet1!$U$3</definedName>
+    <definedName name="_xlchart.v1.45" hidden="1">Sheet1!$U$4:$U$25</definedName>
+    <definedName name="_xlchart.v1.46" hidden="1">Sheet1!$V$3</definedName>
+    <definedName name="_xlchart.v1.47" hidden="1">Sheet1!$V$4:$V$25</definedName>
+    <definedName name="_xlchart.v1.48" hidden="1">Sheet1!$BG$3</definedName>
+    <definedName name="_xlchart.v1.49" hidden="1">Sheet1!$BG$4:$BG$25</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$AU$4:$AU$25</definedName>
+    <definedName name="_xlchart.v1.50" hidden="1">Sheet1!$CQ$3</definedName>
+    <definedName name="_xlchart.v1.51" hidden="1">Sheet1!$CQ$4:$CQ$25</definedName>
+    <definedName name="_xlchart.v1.52" hidden="1">Sheet1!$EA$3</definedName>
+    <definedName name="_xlchart.v1.53" hidden="1">Sheet1!$EA$4:$EA$25</definedName>
+    <definedName name="_xlchart.v1.54" hidden="1">Sheet1!$U$3</definedName>
+    <definedName name="_xlchart.v1.55" hidden="1">Sheet1!$U$4:$U$25</definedName>
+    <definedName name="_xlchart.v1.56" hidden="1">Sheet1!$BE$3</definedName>
+    <definedName name="_xlchart.v1.57" hidden="1">Sheet1!$BE$4:$BE$25</definedName>
+    <definedName name="_xlchart.v1.58" hidden="1">Sheet1!$CO$3</definedName>
+    <definedName name="_xlchart.v1.59" hidden="1">Sheet1!$CO$4:$CO$25</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$AV$3</definedName>
+    <definedName name="_xlchart.v1.60" hidden="1">Sheet1!$DY$3</definedName>
+    <definedName name="_xlchart.v1.61" hidden="1">Sheet1!$DY$4:$DY$25</definedName>
+    <definedName name="_xlchart.v1.62" hidden="1">Sheet1!$S$3</definedName>
+    <definedName name="_xlchart.v1.63" hidden="1">Sheet1!$S$4:$S$25</definedName>
+    <definedName name="_xlchart.v1.64" hidden="1">Sheet1!$AH$3</definedName>
+    <definedName name="_xlchart.v1.65" hidden="1">Sheet1!$AH$4:$AH$25</definedName>
+    <definedName name="_xlchart.v1.66" hidden="1">Sheet1!$BR$3</definedName>
+    <definedName name="_xlchart.v1.67" hidden="1">Sheet1!$BR$4:$BR$25</definedName>
+    <definedName name="_xlchart.v1.68" hidden="1">Sheet1!$DB$3</definedName>
+    <definedName name="_xlchart.v1.69" hidden="1">Sheet1!$DB$4:$DB$25</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$AV$4:$AV$25</definedName>
+    <definedName name="_xlchart.v1.70" hidden="1">Sheet1!$EL$3</definedName>
+    <definedName name="_xlchart.v1.71" hidden="1">Sheet1!$EL$4:$EL$25</definedName>
+    <definedName name="_xlchart.v1.72" hidden="1">Sheet1!$AJ$3</definedName>
+    <definedName name="_xlchart.v1.73" hidden="1">Sheet1!$AJ$4:$AJ$25</definedName>
+    <definedName name="_xlchart.v1.74" hidden="1">Sheet1!$BT$3</definedName>
+    <definedName name="_xlchart.v1.75" hidden="1">Sheet1!$BT$4:$BT$25</definedName>
+    <definedName name="_xlchart.v1.76" hidden="1">Sheet1!$DD$3</definedName>
+    <definedName name="_xlchart.v1.77" hidden="1">Sheet1!$DD$4:$DD$25</definedName>
+    <definedName name="_xlchart.v1.78" hidden="1">Sheet1!$EN$3</definedName>
+    <definedName name="_xlchart.v1.79" hidden="1">Sheet1!$EN$4:$EN$25</definedName>
     <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$BG$3</definedName>
+    <definedName name="_xlchart.v1.80" hidden="1">Sheet1!$AI$3</definedName>
+    <definedName name="_xlchart.v1.81" hidden="1">Sheet1!$AI$4:$AI$25</definedName>
+    <definedName name="_xlchart.v1.82" hidden="1">Sheet1!$AJ$3</definedName>
+    <definedName name="_xlchart.v1.83" hidden="1">Sheet1!$AJ$4:$AJ$25</definedName>
+    <definedName name="_xlchart.v1.84" hidden="1">Sheet1!$AU$3</definedName>
+    <definedName name="_xlchart.v1.85" hidden="1">Sheet1!$AU$4:$AU$25</definedName>
+    <definedName name="_xlchart.v1.86" hidden="1">Sheet1!$AV$3</definedName>
+    <definedName name="_xlchart.v1.87" hidden="1">Sheet1!$AV$4:$AV$25</definedName>
+    <definedName name="_xlchart.v1.88" hidden="1">Sheet1!$BG$3</definedName>
+    <definedName name="_xlchart.v1.89" hidden="1">Sheet1!$BG$4:$BG$25</definedName>
     <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$BG$4:$BG$25</definedName>
+    <definedName name="_xlchart.v1.90" hidden="1">Sheet1!$BH$3</definedName>
+    <definedName name="_xlchart.v1.91" hidden="1">Sheet1!$BH$4:$BH$25</definedName>
+    <definedName name="_xlchart.v1.92" hidden="1">Sheet1!$BS$3</definedName>
+    <definedName name="_xlchart.v1.93" hidden="1">Sheet1!$BS$4:$BS$25</definedName>
+    <definedName name="_xlchart.v1.94" hidden="1">Sheet1!$BT$3</definedName>
+    <definedName name="_xlchart.v1.95" hidden="1">Sheet1!$BT$4:$BT$25</definedName>
+    <definedName name="_xlchart.v1.96" hidden="1">Sheet1!$CE$3</definedName>
+    <definedName name="_xlchart.v1.97" hidden="1">Sheet1!$CE$4:$CE$25</definedName>
+    <definedName name="_xlchart.v1.98" hidden="1">Sheet1!$CF$3</definedName>
+    <definedName name="_xlchart.v1.99" hidden="1">Sheet1!$CF$4:$CF$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -558,7 +654,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -605,7 +701,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5364,122 +5459,122 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.77</cx:f>
+        <cx:f>_xlchart.v1.45</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.79</cx:f>
+        <cx:f>_xlchart.v1.47</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.33</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.35</cx:f>
+        <cx:f>_xlchart.v1.3</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="4">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.37</cx:f>
+        <cx:f>_xlchart.v1.5</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="5">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.39</cx:f>
+        <cx:f>_xlchart.v1.7</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="6">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.41</cx:f>
+        <cx:f>_xlchart.v1.9</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="7">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.43</cx:f>
+        <cx:f>_xlchart.v1.11</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="8">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.45</cx:f>
+        <cx:f>_xlchart.v1.13</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="9">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.47</cx:f>
+        <cx:f>_xlchart.v1.15</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="10">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.49</cx:f>
+        <cx:f>_xlchart.v1.17</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="11">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.51</cx:f>
+        <cx:f>_xlchart.v1.19</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="12">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.53</cx:f>
+        <cx:f>_xlchart.v1.21</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="13">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.55</cx:f>
+        <cx:f>_xlchart.v1.23</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="14">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.57</cx:f>
+        <cx:f>_xlchart.v1.25</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="15">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.59</cx:f>
+        <cx:f>_xlchart.v1.27</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="16">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.61</cx:f>
+        <cx:f>_xlchart.v1.29</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="17">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.63</cx:f>
+        <cx:f>_xlchart.v1.31</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="18">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.65</cx:f>
+        <cx:f>_xlchart.v1.33</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="19">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.67</cx:f>
+        <cx:f>_xlchart.v1.35</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="20">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.69</cx:f>
+        <cx:f>_xlchart.v1.37</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="21">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.71</cx:f>
+        <cx:f>_xlchart.v1.39</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="22">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.73</cx:f>
+        <cx:f>_xlchart.v1.41</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="23">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.75</cx:f>
+        <cx:f>_xlchart.v1.43</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -5517,7 +5612,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{F9C7B960-00DF-46DF-8226-1037739B361D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.76</cx:f>
+              <cx:f>_xlchart.v1.44</cx:f>
               <cx:v>Surface area division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5530,7 +5625,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{B603D70C-3A72-4280-8EA5-E35B3A8F371B}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.78</cx:f>
+              <cx:f>_xlchart.v1.46</cx:f>
               <cx:v>Surface area division bp improvement sd run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5543,7 +5638,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{E180F9C6-9B82-47ED-82D2-ABE3F97580E4}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.32</cx:f>
+              <cx:f>_xlchart.v1.0</cx:f>
               <cx:v>Surface area division sd improvement bp run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5556,7 +5651,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{1A2DCCB6-040F-429A-93AA-5232ABCD77F0}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.34</cx:f>
+              <cx:f>_xlchart.v1.2</cx:f>
               <cx:v>Surface area division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5569,7 +5664,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{83B74E6E-64B3-4EE9-B922-F08CF6274760}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.36</cx:f>
+              <cx:f>_xlchart.v1.4</cx:f>
               <cx:v>Surface area division sd improvement weighted run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5582,7 +5677,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{C325E7ED-CBE7-491D-92EF-A879F5964D24}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.38</cx:f>
+              <cx:f>_xlchart.v1.6</cx:f>
               <cx:v>Surface area division bp improvement weighted run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5595,7 +5690,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{A3F4DEE5-069C-4AA9-AE45-DD53B2EFB7EE}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.40</cx:f>
+              <cx:f>_xlchart.v1.8</cx:f>
               <cx:v>Volume area division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5608,7 +5703,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{130E4B29-CD34-4C7F-AB21-6AE74637EEB9}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.42</cx:f>
+              <cx:f>_xlchart.v1.10</cx:f>
               <cx:v>Volume area division bp improvement sd run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5621,7 +5716,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{C0931B74-7191-44CF-8748-D403A0E4DBBB}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.44</cx:f>
+              <cx:f>_xlchart.v1.12</cx:f>
               <cx:v>Volume area division sd improvement bp run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5634,7 +5729,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{914734F2-4446-445F-B280-09AB701E9E79}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.46</cx:f>
+              <cx:f>_xlchart.v1.14</cx:f>
               <cx:v>Volume area division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5647,7 +5742,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{B1D934F2-2456-4265-AC63-EAA5BC657D96}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.48</cx:f>
+              <cx:f>_xlchart.v1.16</cx:f>
               <cx:v>Volume area division sd improvement weighted run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5660,7 +5755,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{1A873AD5-1F3C-4521-9847-14938DF0C2B1}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.50</cx:f>
+              <cx:f>_xlchart.v1.18</cx:f>
               <cx:v>Volume area division bp improvement weighted run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5673,7 +5768,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{F5F2FB2C-B0B9-4143-98C6-03649858027A}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.52</cx:f>
+              <cx:f>_xlchart.v1.20</cx:f>
               <cx:v>Floor area division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5686,7 +5781,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{C851E9BE-7362-4003-AC79-928BB24AFE7E}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.54</cx:f>
+              <cx:f>_xlchart.v1.22</cx:f>
               <cx:v>Floor area division bp improvement sd run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5699,7 +5794,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{CFFFCFA2-8617-47E2-9D1C-92AA2F6A8894}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.56</cx:f>
+              <cx:f>_xlchart.v1.24</cx:f>
               <cx:v>Floor area division sd improvement bp run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5712,7 +5807,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{B005ED58-0419-4C10-81A0-B2C66550A9D9}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.58</cx:f>
+              <cx:f>_xlchart.v1.26</cx:f>
               <cx:v>Floor area division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5725,7 +5820,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{B91D03C1-EA61-408B-9CCE-D64F2DFF4B97}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.60</cx:f>
+              <cx:f>_xlchart.v1.28</cx:f>
               <cx:v>Floor area division sd improvement weighted run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5738,7 +5833,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{93A40BA7-E3A1-4D76-B948-C44910C6AA91}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.62</cx:f>
+              <cx:f>_xlchart.v1.30</cx:f>
               <cx:v>Floor area division bp improvement weighted run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5751,7 +5846,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000012-12E2-481D-A002-C6AE01E41FF5}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.64</cx:f>
+              <cx:f>_xlchart.v1.32</cx:f>
               <cx:v>No division sd improvement sd run[%] No division bp improvement sd run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5763,7 +5858,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000013-12E2-481D-A002-C6AE01E41FF5}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.66</cx:f>
+              <cx:f>_xlchart.v1.34</cx:f>
               <cx:v>No division bp improvement sd run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5775,7 +5870,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000014-12E2-481D-A002-C6AE01E41FF5}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.68</cx:f>
+              <cx:f>_xlchart.v1.36</cx:f>
               <cx:v>No division sd improvement bp run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5787,7 +5882,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000015-12E2-481D-A002-C6AE01E41FF5}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.70</cx:f>
+              <cx:f>_xlchart.v1.38</cx:f>
               <cx:v>No division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5799,7 +5894,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000016-12E2-481D-A002-C6AE01E41FF5}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.72</cx:f>
+              <cx:f>_xlchart.v1.40</cx:f>
               <cx:v>No division sd improvement weighted run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5811,7 +5906,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{00000017-12E2-481D-A002-C6AE01E41FF5}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.74</cx:f>
+              <cx:f>_xlchart.v1.42</cx:f>
               <cx:v>No division bp improvement weighted run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5889,22 +5984,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.15</cx:f>
+        <cx:f>_xlchart.v1.55</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.9</cx:f>
+        <cx:f>_xlchart.v1.49</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.11</cx:f>
+        <cx:f>_xlchart.v1.51</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.13</cx:f>
+        <cx:f>_xlchart.v1.53</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -5942,7 +6037,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{83960673-2925-49AB-BDE6-6754FDB5B9EF}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.14</cx:f>
+              <cx:f>_xlchart.v1.54</cx:f>
               <cx:v>Surface area division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5955,7 +6050,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{4E62168D-8BD7-4E47-9A24-C2C4C1519AD4}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.8</cx:f>
+              <cx:f>_xlchart.v1.48</cx:f>
               <cx:v>Volume area division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5968,7 +6063,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{21A05520-2063-4E94-AFFB-5BCF34D01FE9}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.10</cx:f>
+              <cx:f>_xlchart.v1.50</cx:f>
               <cx:v>Floor area division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -5988,7 +6083,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{1AB09A40-8190-4BA1-A43E-4976000481CC}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.12</cx:f>
+              <cx:f>_xlchart.v1.52</cx:f>
               <cx:v>No division sd improvement sd run[%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6026,22 +6121,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.17</cx:f>
+        <cx:f>_xlchart.v1.73</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.19</cx:f>
+        <cx:f>_xlchart.v1.75</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.21</cx:f>
+        <cx:f>_xlchart.v1.77</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.23</cx:f>
+        <cx:f>_xlchart.v1.79</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -6079,7 +6174,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{AD4635B5-A96F-4267-B9B2-84E47EE7D6D2}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.16</cx:f>
+              <cx:f>_xlchart.v1.72</cx:f>
               <cx:v>Surface area division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6092,7 +6187,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{F2FFB430-E7E2-4049-AC60-17B7CB20AF56}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.18</cx:f>
+              <cx:f>_xlchart.v1.74</cx:f>
               <cx:v>Volume area division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6105,7 +6200,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{F2EF502C-9F2D-434B-9AC7-FB4A8E5280E0}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.20</cx:f>
+              <cx:f>_xlchart.v1.76</cx:f>
               <cx:v>Floor area division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6118,7 +6213,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{729B749D-D9B5-4A13-90F2-78EEEE1A477C}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.22</cx:f>
+              <cx:f>_xlchart.v1.78</cx:f>
               <cx:v>No division bp improvement bp run [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6149,22 +6244,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.31</cx:f>
+        <cx:f>_xlchart.v1.63</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.25</cx:f>
+        <cx:f>_xlchart.v1.57</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.27</cx:f>
+        <cx:f>_xlchart.v1.59</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.29</cx:f>
+        <cx:f>_xlchart.v1.61</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -6202,7 +6297,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{A1B0B57C-C23B-48C3-91D6-3A5F414E164A}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.30</cx:f>
+              <cx:f>_xlchart.v1.62</cx:f>
               <cx:v>Surface area division sd improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6215,7 +6310,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{D726B8AE-FEEF-47BE-BB9A-6071CB9182D3}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.24</cx:f>
+              <cx:f>_xlchart.v1.56</cx:f>
               <cx:v>Volume area division sd improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6228,7 +6323,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{3DD97FF0-C39B-4D39-8072-336C1B0D183E}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.26</cx:f>
+              <cx:f>_xlchart.v1.58</cx:f>
               <cx:v>Floor area division sd improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6241,7 +6336,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{41BDBAC1-DFAB-4011-B582-DFC80452F05D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.28</cx:f>
+              <cx:f>_xlchart.v1.60</cx:f>
               <cx:v>no division sd improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6272,22 +6367,22 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.65</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="1">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.67</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="2">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.5</cx:f>
+        <cx:f>_xlchart.v1.69</cx:f>
       </cx:numDim>
     </cx:data>
     <cx:data id="3">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.7</cx:f>
+        <cx:f>_xlchart.v1.71</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -6325,7 +6420,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{283FC4D0-F761-4492-A063-F2EB6572FF2E}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.0</cx:f>
+              <cx:f>_xlchart.v1.64</cx:f>
               <cx:v>Surface area division bp improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6338,7 +6433,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{36455C76-3315-42F9-BC82-DE1B4E59BC9D}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.2</cx:f>
+              <cx:f>_xlchart.v1.66</cx:f>
               <cx:v>Volume division bp improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6351,7 +6446,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{F72570FA-6D84-4822-BE04-AA4EE0CFE0A9}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.4</cx:f>
+              <cx:f>_xlchart.v1.68</cx:f>
               <cx:v>Floor area division bp improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6364,7 +6459,7 @@
         <cx:series layoutId="boxWhisker" uniqueId="{9C8B2A34-9A00-4C17-AB7F-84F1BDE26963}">
           <cx:tx>
             <cx:txData>
-              <cx:f>_xlchart.v1.6</cx:f>
+              <cx:f>_xlchart.v1.70</cx:f>
               <cx:v>No division bp improvement last vs. initial [%]</cx:v>
             </cx:txData>
           </cx:tx>
@@ -6390,7 +6485,254 @@
 </cx:chartSpace>
 </file>
 
+<file path=xl/charts/chartEx6.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.101</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.103</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="2">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.105</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="3">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.107</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="4">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.109</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="5">
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.111</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Overvieuw of best vs. initial performance improvement per interation</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+            </a:rPr>
+            <a:t>Overvieuw of best vs. initial performance improvement per interation</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{F5F2FB2C-B0B9-4143-98C6-03649858027A}" formatIdx="12">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.100</cx:f>
+              <cx:v>Floor area division sd improvement sd run[%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{C851E9BE-7362-4003-AC79-928BB24AFE7E}" formatIdx="13">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.102</cx:f>
+              <cx:v>Floor area division bp improvement sd run [%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{CFFFCFA2-8617-47E2-9D1C-92AA2F6A8894}" formatIdx="14">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.104</cx:f>
+              <cx:v>Floor area division sd improvement bp run[%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="2"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{B005ED58-0419-4C10-81A0-B2C66550A9D9}" formatIdx="15">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.106</cx:f>
+              <cx:v>Floor area division bp improvement bp run [%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="3"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{B91D03C1-EA61-408B-9CCE-D64F2DFF4B97}" formatIdx="16">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.108</cx:f>
+              <cx:v>Floor area division sd improvement weighted run[%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="4"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{93A40BA7-E3A1-4D76-B948-C44910C6AA91}" formatIdx="17">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.110</cx:f>
+              <cx:v>Floor area division bp improvement weighted run [%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="5"/>
+          <cx:layoutPr>
+            <cx:visibility meanLine="1" meanMarker="1" nonoutliers="0" outliers="1"/>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0.0500000007"/>
+        <cx:title/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling max="100"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Improvement best vs. inital design performance [%]</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+                </a:rPr>
+                <a:t>Improvement best vs. inital design performance [%]</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="b" align="ctr" overlay="0">
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:solidFill>
+              <a:sysClr val="windowText" lastClr="000000">
+                <a:lumMod val="65000"/>
+                <a:lumOff val="35000"/>
+              </a:sysClr>
+            </a:solidFill>
+            <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+          </a:endParaRPr>
+        </a:p>
+      </cx:txPr>
+    </cx:legend>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -7265,6 +7607,521 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="373">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="373">
   <cs:axisTitle>
@@ -11678,8 +12535,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="9782173" y="7229475"/>
-              <a:ext cx="10925177" cy="8601075"/>
+              <a:off x="9791698" y="7277100"/>
+              <a:ext cx="10934702" cy="8679180"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -11756,8 +12613,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="20983572" y="7222806"/>
-              <a:ext cx="3158493" cy="5083494"/>
+              <a:off x="21008337" y="7264716"/>
+              <a:ext cx="3150873" cy="5125404"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -11834,8 +12691,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="24240174" y="7209472"/>
-              <a:ext cx="2904171" cy="5066348"/>
+              <a:off x="24253509" y="7253287"/>
+              <a:ext cx="2909886" cy="5112068"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -11912,8 +12769,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="27410092" y="7222806"/>
-              <a:ext cx="3336608" cy="4961574"/>
+              <a:off x="27429142" y="7264716"/>
+              <a:ext cx="3332798" cy="5005389"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -11990,8 +12847,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="30861953" y="7203757"/>
-              <a:ext cx="3481388" cy="4957763"/>
+              <a:off x="30884813" y="7249477"/>
+              <a:ext cx="3469958" cy="5001578"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -12163,6 +13020,84 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>243840</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>396240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>47</xdr:col>
+      <xdr:colOff>998220</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Chart 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57FB606E-E16B-49AB-A104-FDA9ED20A09D}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="34709100" y="7711440"/>
+              <a:ext cx="6705600" cy="4381500"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-NL" sz="1100"/>
+                <a:t>This chart isn't available in your version of Excel.
+Editing this shape or saving this workbook into a different file format will permanently break the chart.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -24734,19 +25669,19 @@
       </c>
     </row>
     <row r="27" spans="1:194" x14ac:dyDescent="0.3">
-      <c r="AR27" s="32"/>
+      <c r="AR27"/>
     </row>
     <row r="28" spans="1:194" x14ac:dyDescent="0.3">
-      <c r="AR28" s="32"/>
+      <c r="AR28"/>
     </row>
     <row r="29" spans="1:194" x14ac:dyDescent="0.3">
-      <c r="AR29" s="32"/>
+      <c r="AR29"/>
     </row>
     <row r="30" spans="1:194" x14ac:dyDescent="0.3">
       <c r="C30" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="AR30" s="32"/>
+      <c r="AR30"/>
     </row>
     <row r="31" spans="1:194" ht="87" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="20" t="s">
@@ -24779,7 +25714,7 @@
       <c r="K31" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="AR31" s="32"/>
+      <c r="AR31"/>
     </row>
     <row r="32" spans="1:194" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
@@ -24820,7 +25755,7 @@
         <f>SUM(H32:H34)</f>
         <v>24.894601099027803</v>
       </c>
-      <c r="AR32" s="32"/>
+      <c r="AR32"/>
     </row>
     <row r="33" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
@@ -24830,30 +25765,30 @@
         <v>10</v>
       </c>
       <c r="C33" s="12">
-        <f>AE26</f>
+        <f t="shared" ref="C33:H33" si="16">AE26</f>
         <v>8.5909090909090917</v>
       </c>
       <c r="D33" s="2">
-        <f>AF26</f>
+        <f t="shared" si="16"/>
         <v>8.3181818181818183</v>
       </c>
       <c r="E33" s="19">
-        <f>AG26</f>
+        <f t="shared" si="16"/>
         <v>40.439780394979771</v>
       </c>
       <c r="F33" s="19">
-        <f>AH26</f>
+        <f t="shared" si="16"/>
         <v>9.7096637217398563</v>
       </c>
       <c r="G33" s="19">
-        <f>AI26</f>
+        <f t="shared" si="16"/>
         <v>55.423737385769485</v>
       </c>
       <c r="H33" s="19">
-        <f>AJ26</f>
+        <f t="shared" si="16"/>
         <v>12.658654773907944</v>
       </c>
-      <c r="AR33" s="32"/>
+      <c r="AR33"/>
     </row>
     <row r="34" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
@@ -24863,30 +25798,30 @@
         <v>47</v>
       </c>
       <c r="C34" s="23">
-        <f>AQ26</f>
+        <f t="shared" ref="C34:H34" si="17">AQ26</f>
         <v>8.9047619047619051</v>
       </c>
       <c r="D34" s="24">
-        <f>AR26</f>
+        <f t="shared" si="17"/>
         <v>8.5714285714285712</v>
       </c>
       <c r="E34" s="24">
-        <f>AS26</f>
+        <f t="shared" si="17"/>
         <v>-223.05743844633557</v>
       </c>
       <c r="F34" s="24">
-        <f>AT26</f>
+        <f t="shared" si="17"/>
         <v>5.4043583399949693</v>
       </c>
       <c r="G34" s="24">
-        <f>AU26</f>
+        <f t="shared" si="17"/>
         <v>53.043073412372692</v>
       </c>
       <c r="H34" s="24">
-        <f>AV26</f>
+        <f t="shared" si="17"/>
         <v>9.4130240727579739</v>
       </c>
-      <c r="AR34" s="32"/>
+      <c r="AR34"/>
     </row>
     <row r="35" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
@@ -24896,38 +25831,38 @@
         <v>9</v>
       </c>
       <c r="C35" s="12">
-        <f>BC26</f>
+        <f t="shared" ref="C35:H35" si="18">BC26</f>
         <v>6.5714285714285712</v>
       </c>
       <c r="D35" s="2">
-        <f>BD26</f>
+        <f t="shared" si="18"/>
         <v>4.1904761904761907</v>
       </c>
       <c r="E35" s="2">
-        <f>BE26</f>
+        <f t="shared" si="18"/>
         <v>0.76651693491220829</v>
       </c>
       <c r="F35" s="2">
-        <f>BF26</f>
+        <f t="shared" si="18"/>
         <v>-6.6450954859109128</v>
       </c>
       <c r="G35" s="2">
-        <f>BG26</f>
+        <f t="shared" si="18"/>
         <v>47.141485340541273</v>
       </c>
       <c r="H35" s="2">
-        <f>BH26</f>
+        <f t="shared" si="18"/>
         <v>3.663267406213345</v>
       </c>
       <c r="J35" s="2">
-        <f t="shared" ref="J35:K35" si="16">SUM(G35:G37)</f>
+        <f t="shared" ref="J35:K35" si="19">SUM(G35:G37)</f>
         <v>154.25692679726859</v>
       </c>
       <c r="K35" s="2">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>12.695359632715126</v>
       </c>
-      <c r="AR35" s="32"/>
+      <c r="AR35"/>
     </row>
     <row r="36" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
@@ -24937,30 +25872,30 @@
         <v>10</v>
       </c>
       <c r="C36" s="12">
-        <f>BO26</f>
+        <f t="shared" ref="C36:H36" si="20">BO26</f>
         <v>8.7142857142857135</v>
       </c>
       <c r="D36" s="2">
-        <f>BP26</f>
+        <f t="shared" si="20"/>
         <v>5.8571428571428568</v>
       </c>
       <c r="E36" s="19">
-        <f>BQ26</f>
+        <f t="shared" si="20"/>
         <v>39.732376293897993</v>
       </c>
       <c r="F36" s="2">
-        <f>BR26</f>
+        <f t="shared" si="20"/>
         <v>-8.7762886438604806</v>
       </c>
       <c r="G36" s="19">
-        <f>BS26</f>
+        <f t="shared" si="20"/>
         <v>55.277695216693289</v>
       </c>
       <c r="H36" s="19">
-        <f>BT26</f>
+        <f t="shared" si="20"/>
         <v>5.0872879859785387</v>
       </c>
-      <c r="AR36" s="32"/>
+      <c r="AR36"/>
     </row>
     <row r="37" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A37" s="15" t="s">
@@ -24970,30 +25905,30 @@
         <v>47</v>
       </c>
       <c r="C37" s="23">
-        <f>CA26</f>
+        <f t="shared" ref="C37:H37" si="21">CA26</f>
         <v>9.0952380952380949</v>
       </c>
       <c r="D37" s="24">
-        <f>CB26</f>
+        <f t="shared" si="21"/>
         <v>5.666666666666667</v>
       </c>
       <c r="E37" s="24">
-        <f>CC26</f>
+        <f t="shared" si="21"/>
         <v>33.275692830607056</v>
       </c>
       <c r="F37" s="25">
-        <f>CD26</f>
+        <f t="shared" si="21"/>
         <v>-1.3645437121129322</v>
       </c>
       <c r="G37" s="24">
-        <f>CE26</f>
+        <f t="shared" si="21"/>
         <v>51.837746240034015</v>
       </c>
       <c r="H37" s="24">
-        <f>CF26</f>
+        <f t="shared" si="21"/>
         <v>3.9448042405232422</v>
       </c>
-      <c r="AR37" s="32"/>
+      <c r="AR37"/>
     </row>
     <row r="38" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
@@ -25003,38 +25938,38 @@
         <v>9</v>
       </c>
       <c r="C38" s="12">
-        <f>BC26</f>
+        <f t="shared" ref="C38:H38" si="22">BC26</f>
         <v>6.5714285714285712</v>
       </c>
       <c r="D38" s="2">
-        <f>BD26</f>
+        <f t="shared" si="22"/>
         <v>4.1904761904761907</v>
       </c>
       <c r="E38" s="2">
-        <f>BE26</f>
+        <f t="shared" si="22"/>
         <v>0.76651693491220829</v>
       </c>
       <c r="F38" s="2">
-        <f>BF26</f>
+        <f t="shared" si="22"/>
         <v>-6.6450954859109128</v>
       </c>
       <c r="G38" s="2">
-        <f>BG26</f>
+        <f t="shared" si="22"/>
         <v>47.141485340541273</v>
       </c>
       <c r="H38" s="2">
-        <f>BH26</f>
+        <f t="shared" si="22"/>
         <v>3.663267406213345</v>
       </c>
       <c r="J38" s="2">
-        <f t="shared" ref="J38:K38" si="17">SUM(G38:G40)</f>
+        <f t="shared" ref="J38:K38" si="23">SUM(G38:G40)</f>
         <v>153.37307648070816</v>
       </c>
       <c r="K38" s="2">
-        <f t="shared" si="17"/>
+        <f t="shared" si="23"/>
         <v>26.58250332580414</v>
       </c>
-      <c r="AR38" s="32"/>
+      <c r="AR38"/>
     </row>
     <row r="39" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
@@ -25044,30 +25979,30 @@
         <v>10</v>
       </c>
       <c r="C39" s="12">
-        <f>CY26</f>
+        <f t="shared" ref="C39:H39" si="24">CY26</f>
         <v>9.8000000000000007</v>
       </c>
       <c r="D39" s="2">
-        <f>CZ26</f>
+        <f t="shared" si="24"/>
         <v>9.4499999999999993</v>
       </c>
       <c r="E39" s="19">
-        <f>DA26</f>
+        <f t="shared" si="24"/>
         <v>32.15704819007636</v>
       </c>
       <c r="F39" s="19">
-        <f>DB26</f>
+        <f t="shared" si="24"/>
         <v>12.619150131104394</v>
       </c>
       <c r="G39" s="19">
-        <f>DC26</f>
+        <f t="shared" si="24"/>
         <v>54.986539071972899</v>
       </c>
       <c r="H39" s="19">
-        <f>DD26</f>
+        <f t="shared" si="24"/>
         <v>14.150666447131602</v>
       </c>
-      <c r="AR39" s="32"/>
+      <c r="AR39"/>
     </row>
     <row r="40" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A40" s="15" t="s">
@@ -25077,30 +26012,30 @@
         <v>47</v>
       </c>
       <c r="C40" s="12">
-        <f>DK26</f>
+        <f t="shared" ref="C40:H40" si="25">DK26</f>
         <v>8.8636363636363633</v>
       </c>
       <c r="D40" s="2">
-        <f>DL26</f>
+        <f t="shared" si="25"/>
         <v>8.3181818181818183</v>
       </c>
       <c r="E40" s="2">
-        <f>DM26</f>
+        <f t="shared" si="25"/>
         <v>23.147866593745615</v>
       </c>
       <c r="F40" s="2">
-        <f>DN26</f>
+        <f t="shared" si="25"/>
         <v>3.0430744679493715</v>
       </c>
       <c r="G40" s="2">
-        <f>DO26</f>
+        <f t="shared" si="25"/>
         <v>51.245052068193985</v>
       </c>
       <c r="H40" s="2">
-        <f>DP26</f>
+        <f t="shared" si="25"/>
         <v>8.7685694724591929</v>
       </c>
-      <c r="AR40" s="32"/>
+      <c r="AR40"/>
     </row>
     <row r="41" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -25110,38 +26045,38 @@
         <v>9</v>
       </c>
       <c r="C41" s="28">
-        <f>DW26</f>
+        <f t="shared" ref="C41:H41" si="26">DW26</f>
         <v>5.8421052631578947</v>
       </c>
       <c r="D41" s="29">
-        <f>DX26</f>
+        <f t="shared" si="26"/>
         <v>3.3157894736842106</v>
       </c>
       <c r="E41" s="29">
-        <f>DY26</f>
+        <f t="shared" si="26"/>
         <v>-22.91784086653195</v>
       </c>
       <c r="F41" s="29">
-        <f>DZ26</f>
+        <f t="shared" si="26"/>
         <v>-9.8540669385721245</v>
       </c>
       <c r="G41" s="29">
-        <f>EA26</f>
+        <f t="shared" si="26"/>
         <v>42.217156080341219</v>
       </c>
       <c r="H41" s="29">
-        <f>EB26</f>
+        <f t="shared" si="26"/>
         <v>1.5926033480137503</v>
       </c>
       <c r="J41" s="2">
-        <f t="shared" ref="J41:K41" si="18">SUM(G41:G43)</f>
+        <f t="shared" ref="J41:K41" si="27">SUM(G41:G43)</f>
         <v>146.97507146087787</v>
       </c>
       <c r="K41" s="2">
-        <f t="shared" si="18"/>
+        <f t="shared" si="27"/>
         <v>21.800829385424386</v>
       </c>
-      <c r="AR41" s="32"/>
+      <c r="AR41"/>
     </row>
     <row r="42" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -25151,30 +26086,30 @@
         <v>10</v>
       </c>
       <c r="C42" s="12">
-        <f>EI26</f>
+        <f t="shared" ref="C42:H42" si="28">EI26</f>
         <v>8.3809523809523814</v>
       </c>
       <c r="D42" s="2">
-        <f>EJ26</f>
+        <f t="shared" si="28"/>
         <v>7.8571428571428568</v>
       </c>
       <c r="E42" s="19">
-        <f>EK26</f>
+        <f t="shared" si="28"/>
         <v>35.20940121009717</v>
       </c>
       <c r="F42" s="19">
-        <f>EL26</f>
+        <f t="shared" si="28"/>
         <v>8.6419893121444833</v>
       </c>
       <c r="G42" s="19">
-        <f>EM26</f>
+        <f t="shared" si="28"/>
         <v>56.388780222842698</v>
       </c>
       <c r="H42" s="19">
-        <f>EN26</f>
+        <f t="shared" si="28"/>
         <v>13.088908709192744</v>
       </c>
-      <c r="AR42" s="32"/>
+      <c r="AR42"/>
     </row>
     <row r="43" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A43" s="15" t="s">
@@ -25184,30 +26119,30 @@
         <v>47</v>
       </c>
       <c r="C43" s="23">
-        <f>EU26</f>
+        <f t="shared" ref="C43:H43" si="29">EU26</f>
         <v>8.2272727272727266</v>
       </c>
       <c r="D43" s="2">
-        <f>EV26</f>
+        <f t="shared" si="29"/>
         <v>4.9090909090909092</v>
       </c>
       <c r="E43" s="2">
-        <f>EW26</f>
+        <f t="shared" si="29"/>
         <v>-12.628337411455288</v>
       </c>
       <c r="F43" s="2">
-        <f>EX26</f>
+        <f t="shared" si="29"/>
         <v>-4.2775720398322941</v>
       </c>
       <c r="G43" s="2">
-        <f>EY26</f>
+        <f t="shared" si="29"/>
         <v>48.369135157693968</v>
       </c>
       <c r="H43" s="2">
-        <f>EZ26</f>
+        <f t="shared" si="29"/>
         <v>7.1193173282178925</v>
       </c>
-      <c r="AR43" s="32"/>
+      <c r="AR43"/>
     </row>
     <row r="44" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
@@ -25217,38 +26152,38 @@
         <v>9</v>
       </c>
       <c r="C44" s="28">
-        <f>FI26</f>
+        <f t="shared" ref="C44:H44" si="30">FI26</f>
         <v>6.3636363636363633</v>
       </c>
       <c r="D44" s="29">
-        <f>FJ26</f>
+        <f t="shared" si="30"/>
         <v>1.3636363636363635</v>
       </c>
       <c r="E44" s="29">
-        <f>FK26</f>
+        <f t="shared" si="30"/>
         <v>-24698.287646488167</v>
       </c>
       <c r="F44" s="29">
-        <f>FL26</f>
+        <f t="shared" si="30"/>
         <v>-13.180752345605809</v>
       </c>
       <c r="G44" s="29">
-        <f>FM26</f>
+        <f t="shared" si="30"/>
         <v>31.445755964131276</v>
       </c>
       <c r="H44" s="29">
-        <f>FN26</f>
+        <f t="shared" si="30"/>
         <v>1.3025099931351602</v>
       </c>
       <c r="J44" s="2">
-        <f t="shared" ref="J44" si="19">SUM(G44:G46)</f>
+        <f t="shared" ref="J44" si="31">SUM(G44:G46)</f>
         <v>111.04001470439067</v>
       </c>
       <c r="K44" s="2">
-        <f t="shared" ref="K44" si="20">SUM(H44:H46)</f>
+        <f t="shared" ref="K44" si="32">SUM(H44:H46)</f>
         <v>11.097124795271647</v>
       </c>
-      <c r="AR44" s="32"/>
+      <c r="AR44"/>
     </row>
     <row r="45" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -25262,26 +26197,26 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="D45" s="2">
-        <f t="shared" ref="D45:H45" si="21">FV26</f>
+        <f t="shared" ref="D45:H45" si="33">FV26</f>
         <v>3.8666666666666667</v>
       </c>
       <c r="E45" s="19">
-        <f t="shared" si="21"/>
+        <f t="shared" si="33"/>
         <v>-123.69330695574695</v>
       </c>
       <c r="F45" s="19">
-        <f t="shared" si="21"/>
+        <f t="shared" si="33"/>
         <v>0.16752662829177467</v>
       </c>
       <c r="G45" s="19">
-        <f t="shared" si="21"/>
+        <f t="shared" si="33"/>
         <v>50.504698489128558</v>
       </c>
       <c r="H45" s="19">
-        <f t="shared" si="21"/>
+        <f t="shared" si="33"/>
         <v>5.6349562940793909</v>
       </c>
-      <c r="AR45" s="32"/>
+      <c r="AR45"/>
     </row>
     <row r="46" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
@@ -25295,1859 +26230,1859 @@
         <v>6.333333333333333</v>
       </c>
       <c r="D46" s="24">
-        <f t="shared" ref="D46:H46" si="22">GH26</f>
+        <f t="shared" ref="D46:H46" si="34">GH26</f>
         <v>1.9333333333333333</v>
       </c>
       <c r="E46" s="24">
-        <f t="shared" si="22"/>
+        <f t="shared" si="34"/>
         <v>-2057.4406516906602</v>
       </c>
       <c r="F46" s="24">
-        <f t="shared" si="22"/>
+        <f t="shared" si="34"/>
         <v>-3.1680569829254148</v>
       </c>
       <c r="G46" s="24">
-        <f t="shared" si="22"/>
+        <f t="shared" si="34"/>
         <v>29.089560251130827</v>
       </c>
       <c r="H46" s="24">
-        <f t="shared" si="22"/>
+        <f t="shared" si="34"/>
         <v>4.1596585080570954</v>
       </c>
-      <c r="AR46" s="32"/>
+      <c r="AR46"/>
     </row>
     <row r="47" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="AR47" s="32"/>
+      <c r="AR47"/>
     </row>
     <row r="48" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="AR48" s="32"/>
+      <c r="AR48"/>
     </row>
     <row r="49" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR49" s="32"/>
+      <c r="AR49"/>
     </row>
     <row r="50" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR50" s="32"/>
+      <c r="AR50"/>
     </row>
     <row r="51" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR51" s="32"/>
+      <c r="AR51"/>
     </row>
     <row r="52" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR52" s="32"/>
+      <c r="AR52"/>
     </row>
     <row r="53" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR53" s="32"/>
+      <c r="AR53"/>
     </row>
     <row r="54" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR54" s="32"/>
+      <c r="AR54"/>
     </row>
     <row r="55" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR55" s="32"/>
+      <c r="AR55"/>
     </row>
     <row r="56" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR56" s="32"/>
+      <c r="AR56"/>
     </row>
     <row r="57" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR57" s="32"/>
+      <c r="AR57"/>
     </row>
     <row r="58" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR58" s="32"/>
+      <c r="AR58"/>
     </row>
     <row r="59" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR59" s="32"/>
+      <c r="AR59"/>
     </row>
     <row r="60" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR60" s="32"/>
+      <c r="AR60"/>
     </row>
     <row r="61" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR61" s="32"/>
+      <c r="AR61"/>
     </row>
     <row r="62" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR62" s="32"/>
+      <c r="AR62"/>
     </row>
     <row r="63" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR63" s="32"/>
+      <c r="AR63"/>
     </row>
     <row r="64" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR64" s="32"/>
+      <c r="AR64"/>
     </row>
     <row r="65" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR65" s="32"/>
+      <c r="AR65"/>
     </row>
     <row r="66" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR66" s="32"/>
+      <c r="AR66"/>
     </row>
     <row r="67" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR67" s="32"/>
+      <c r="AR67"/>
     </row>
     <row r="68" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR68" s="32"/>
+      <c r="AR68"/>
     </row>
     <row r="69" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR69" s="32"/>
+      <c r="AR69"/>
     </row>
     <row r="70" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR70" s="32"/>
+      <c r="AR70"/>
     </row>
     <row r="71" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR71" s="32"/>
+      <c r="AR71"/>
     </row>
     <row r="72" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR72" s="32"/>
+      <c r="AR72"/>
     </row>
     <row r="73" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR73" s="32"/>
+      <c r="AR73"/>
     </row>
     <row r="74" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR74" s="32"/>
+      <c r="AR74"/>
     </row>
     <row r="75" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR75" s="32"/>
+      <c r="AR75"/>
     </row>
     <row r="76" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR76" s="32"/>
+      <c r="AR76"/>
     </row>
     <row r="77" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR77" s="32"/>
+      <c r="AR77"/>
     </row>
     <row r="78" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR78" s="32"/>
+      <c r="AR78"/>
     </row>
     <row r="79" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR79" s="32"/>
+      <c r="AR79"/>
     </row>
     <row r="80" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR80" s="32"/>
+      <c r="AR80"/>
     </row>
     <row r="81" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR81" s="32"/>
+      <c r="AR81"/>
     </row>
     <row r="82" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR82" s="32"/>
+      <c r="AR82"/>
     </row>
     <row r="83" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR83" s="32"/>
+      <c r="AR83"/>
     </row>
     <row r="84" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR84" s="32"/>
+      <c r="AR84"/>
     </row>
     <row r="85" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR85" s="32"/>
+      <c r="AR85"/>
     </row>
     <row r="86" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR86" s="32"/>
+      <c r="AR86"/>
     </row>
     <row r="87" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR87" s="32"/>
+      <c r="AR87"/>
     </row>
     <row r="88" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR88" s="32"/>
+      <c r="AR88"/>
     </row>
     <row r="89" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR89" s="32"/>
+      <c r="AR89"/>
     </row>
     <row r="90" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR90" s="32"/>
+      <c r="AR90"/>
     </row>
     <row r="91" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR91" s="32"/>
+      <c r="AR91"/>
     </row>
     <row r="92" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR92" s="32"/>
+      <c r="AR92"/>
     </row>
     <row r="93" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR93" s="32"/>
+      <c r="AR93"/>
     </row>
     <row r="94" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR94" s="32"/>
+      <c r="AR94"/>
     </row>
     <row r="95" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR95" s="32"/>
+      <c r="AR95"/>
     </row>
     <row r="96" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR96" s="32"/>
+      <c r="AR96"/>
     </row>
     <row r="97" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR97" s="32"/>
+      <c r="AR97"/>
     </row>
     <row r="98" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR98" s="32"/>
+      <c r="AR98"/>
     </row>
     <row r="99" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR99" s="32"/>
+      <c r="AR99"/>
     </row>
     <row r="100" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR100" s="32"/>
+      <c r="AR100"/>
     </row>
     <row r="101" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR101" s="32"/>
+      <c r="AR101"/>
     </row>
     <row r="102" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR102" s="32"/>
+      <c r="AR102"/>
     </row>
     <row r="103" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR103" s="32"/>
+      <c r="AR103"/>
     </row>
     <row r="104" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR104" s="32"/>
+      <c r="AR104"/>
     </row>
     <row r="105" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR105" s="32"/>
+      <c r="AR105"/>
     </row>
     <row r="106" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR106" s="32"/>
+      <c r="AR106"/>
     </row>
     <row r="107" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR107" s="32"/>
+      <c r="AR107"/>
     </row>
     <row r="108" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR108" s="32"/>
+      <c r="AR108"/>
     </row>
     <row r="109" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR109" s="32"/>
+      <c r="AR109"/>
     </row>
     <row r="110" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR110" s="32"/>
+      <c r="AR110"/>
     </row>
     <row r="111" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR111" s="32"/>
+      <c r="AR111"/>
     </row>
     <row r="112" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR112" s="32"/>
+      <c r="AR112"/>
     </row>
     <row r="113" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR113" s="32"/>
+      <c r="AR113"/>
     </row>
     <row r="114" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR114" s="32"/>
+      <c r="AR114"/>
     </row>
     <row r="115" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR115" s="32"/>
+      <c r="AR115"/>
     </row>
     <row r="116" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR116" s="32"/>
+      <c r="AR116"/>
     </row>
     <row r="117" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR117" s="32"/>
+      <c r="AR117"/>
     </row>
     <row r="118" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR118" s="32"/>
+      <c r="AR118"/>
     </row>
     <row r="119" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR119" s="32"/>
+      <c r="AR119"/>
     </row>
     <row r="120" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR120" s="32"/>
+      <c r="AR120"/>
     </row>
     <row r="121" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR121" s="32"/>
+      <c r="AR121"/>
     </row>
     <row r="122" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR122" s="32"/>
+      <c r="AR122"/>
     </row>
     <row r="123" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR123" s="32"/>
+      <c r="AR123"/>
     </row>
     <row r="124" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR124" s="32"/>
+      <c r="AR124"/>
     </row>
     <row r="125" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR125" s="32"/>
+      <c r="AR125"/>
     </row>
     <row r="126" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR126" s="32"/>
+      <c r="AR126"/>
     </row>
     <row r="127" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR127" s="32"/>
+      <c r="AR127"/>
     </row>
     <row r="128" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR128" s="32"/>
+      <c r="AR128"/>
     </row>
     <row r="129" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR129" s="32"/>
+      <c r="AR129"/>
     </row>
     <row r="130" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR130" s="32"/>
+      <c r="AR130"/>
     </row>
     <row r="131" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR131" s="32"/>
+      <c r="AR131"/>
     </row>
     <row r="132" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR132" s="32"/>
+      <c r="AR132"/>
     </row>
     <row r="133" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR133" s="32"/>
+      <c r="AR133"/>
     </row>
     <row r="134" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR134" s="32"/>
+      <c r="AR134"/>
     </row>
     <row r="135" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR135" s="32"/>
+      <c r="AR135"/>
     </row>
     <row r="136" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR136" s="32"/>
+      <c r="AR136"/>
     </row>
     <row r="137" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR137" s="32"/>
+      <c r="AR137"/>
     </row>
     <row r="138" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR138" s="32"/>
+      <c r="AR138"/>
     </row>
     <row r="139" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR139" s="32"/>
+      <c r="AR139"/>
     </row>
     <row r="140" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR140" s="32"/>
+      <c r="AR140"/>
     </row>
     <row r="141" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR141" s="32"/>
+      <c r="AR141"/>
     </row>
     <row r="142" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR142" s="32"/>
+      <c r="AR142"/>
     </row>
     <row r="143" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR143" s="32"/>
+      <c r="AR143"/>
     </row>
     <row r="144" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR144" s="32"/>
+      <c r="AR144"/>
     </row>
     <row r="145" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR145" s="32"/>
+      <c r="AR145"/>
     </row>
     <row r="146" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR146" s="32"/>
+      <c r="AR146"/>
     </row>
     <row r="147" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR147" s="32"/>
+      <c r="AR147"/>
     </row>
     <row r="148" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR148" s="32"/>
+      <c r="AR148"/>
     </row>
     <row r="149" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR149" s="32"/>
+      <c r="AR149"/>
     </row>
     <row r="150" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR150" s="32"/>
+      <c r="AR150"/>
     </row>
     <row r="151" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR151" s="32"/>
+      <c r="AR151"/>
     </row>
     <row r="152" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR152" s="32"/>
+      <c r="AR152"/>
     </row>
     <row r="153" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR153" s="32"/>
+      <c r="AR153"/>
     </row>
     <row r="154" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR154" s="32"/>
+      <c r="AR154"/>
     </row>
     <row r="155" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR155" s="32"/>
+      <c r="AR155"/>
     </row>
     <row r="156" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR156" s="32"/>
+      <c r="AR156"/>
     </row>
     <row r="157" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR157" s="32"/>
+      <c r="AR157"/>
     </row>
     <row r="158" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR158" s="32"/>
+      <c r="AR158"/>
     </row>
     <row r="159" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR159" s="32"/>
+      <c r="AR159"/>
     </row>
     <row r="160" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR160" s="32"/>
+      <c r="AR160"/>
     </row>
     <row r="161" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR161" s="32"/>
+      <c r="AR161"/>
     </row>
     <row r="162" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR162" s="32"/>
+      <c r="AR162"/>
     </row>
     <row r="163" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR163" s="32"/>
+      <c r="AR163"/>
     </row>
     <row r="164" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR164" s="32"/>
+      <c r="AR164"/>
     </row>
     <row r="165" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR165" s="32"/>
+      <c r="AR165"/>
     </row>
     <row r="166" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR166" s="32"/>
+      <c r="AR166"/>
     </row>
     <row r="167" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR167" s="32"/>
+      <c r="AR167"/>
     </row>
     <row r="168" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR168" s="32"/>
+      <c r="AR168"/>
     </row>
     <row r="169" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR169" s="32"/>
+      <c r="AR169"/>
     </row>
     <row r="170" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR170" s="32"/>
+      <c r="AR170"/>
     </row>
     <row r="171" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR171" s="32"/>
+      <c r="AR171"/>
     </row>
     <row r="172" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR172" s="32"/>
+      <c r="AR172"/>
     </row>
     <row r="173" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR173" s="32"/>
+      <c r="AR173"/>
     </row>
     <row r="174" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR174" s="32"/>
+      <c r="AR174"/>
     </row>
     <row r="175" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR175" s="32"/>
+      <c r="AR175"/>
     </row>
     <row r="176" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR176" s="32"/>
+      <c r="AR176"/>
     </row>
     <row r="177" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR177" s="32"/>
+      <c r="AR177"/>
     </row>
     <row r="178" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR178" s="32"/>
+      <c r="AR178"/>
     </row>
     <row r="179" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR179" s="32"/>
+      <c r="AR179"/>
     </row>
     <row r="180" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR180" s="32"/>
+      <c r="AR180"/>
     </row>
     <row r="181" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR181" s="32"/>
+      <c r="AR181"/>
     </row>
     <row r="182" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR182" s="32"/>
+      <c r="AR182"/>
     </row>
     <row r="183" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR183" s="32"/>
+      <c r="AR183"/>
     </row>
     <row r="184" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR184" s="32"/>
+      <c r="AR184"/>
     </row>
     <row r="185" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR185" s="32"/>
+      <c r="AR185"/>
     </row>
     <row r="186" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR186" s="32"/>
+      <c r="AR186"/>
     </row>
     <row r="187" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR187" s="32"/>
+      <c r="AR187"/>
     </row>
     <row r="188" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR188" s="32"/>
+      <c r="AR188"/>
     </row>
     <row r="189" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR189" s="32"/>
+      <c r="AR189"/>
     </row>
     <row r="190" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR190" s="32"/>
+      <c r="AR190"/>
     </row>
     <row r="191" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR191" s="32"/>
+      <c r="AR191"/>
     </row>
     <row r="192" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR192" s="32"/>
+      <c r="AR192"/>
     </row>
     <row r="193" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR193" s="32"/>
+      <c r="AR193"/>
     </row>
     <row r="194" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR194" s="32"/>
+      <c r="AR194"/>
     </row>
     <row r="195" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR195" s="32"/>
+      <c r="AR195"/>
     </row>
     <row r="196" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR196" s="32"/>
+      <c r="AR196"/>
     </row>
     <row r="197" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR197" s="32"/>
+      <c r="AR197"/>
     </row>
     <row r="198" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR198" s="32"/>
+      <c r="AR198"/>
     </row>
     <row r="199" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR199" s="32"/>
+      <c r="AR199"/>
     </row>
     <row r="200" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR200" s="32"/>
+      <c r="AR200"/>
     </row>
     <row r="201" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR201" s="32"/>
+      <c r="AR201"/>
     </row>
     <row r="202" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR202" s="32"/>
+      <c r="AR202"/>
     </row>
     <row r="203" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR203" s="32"/>
+      <c r="AR203"/>
     </row>
     <row r="204" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR204" s="32"/>
+      <c r="AR204"/>
     </row>
     <row r="205" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR205" s="32"/>
+      <c r="AR205"/>
     </row>
     <row r="206" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR206" s="32"/>
+      <c r="AR206"/>
     </row>
     <row r="207" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR207" s="32"/>
+      <c r="AR207"/>
     </row>
     <row r="208" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR208" s="32"/>
+      <c r="AR208"/>
     </row>
     <row r="209" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR209" s="32"/>
+      <c r="AR209"/>
     </row>
     <row r="210" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR210" s="32"/>
+      <c r="AR210"/>
     </row>
     <row r="211" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR211" s="32"/>
+      <c r="AR211"/>
     </row>
     <row r="212" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR212" s="32"/>
+      <c r="AR212"/>
     </row>
     <row r="213" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR213" s="32"/>
+      <c r="AR213"/>
     </row>
     <row r="214" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR214" s="32"/>
+      <c r="AR214"/>
     </row>
     <row r="215" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR215" s="32"/>
+      <c r="AR215"/>
     </row>
     <row r="216" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR216" s="32"/>
+      <c r="AR216"/>
     </row>
     <row r="217" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR217" s="32"/>
+      <c r="AR217"/>
     </row>
     <row r="218" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR218" s="32"/>
+      <c r="AR218"/>
     </row>
     <row r="219" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR219" s="32"/>
+      <c r="AR219"/>
     </row>
     <row r="220" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR220" s="32"/>
+      <c r="AR220"/>
     </row>
     <row r="221" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR221" s="32"/>
+      <c r="AR221"/>
     </row>
     <row r="222" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR222" s="32"/>
+      <c r="AR222"/>
     </row>
     <row r="223" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR223" s="32"/>
+      <c r="AR223"/>
     </row>
     <row r="224" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR224" s="32"/>
+      <c r="AR224"/>
     </row>
     <row r="225" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR225" s="32"/>
+      <c r="AR225"/>
     </row>
     <row r="226" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR226" s="32"/>
+      <c r="AR226"/>
     </row>
     <row r="227" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR227" s="32"/>
+      <c r="AR227"/>
     </row>
     <row r="228" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR228" s="32"/>
+      <c r="AR228"/>
     </row>
     <row r="229" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR229" s="32"/>
+      <c r="AR229"/>
     </row>
     <row r="230" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR230" s="32"/>
+      <c r="AR230"/>
     </row>
     <row r="231" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR231" s="32"/>
+      <c r="AR231"/>
     </row>
     <row r="232" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR232" s="32"/>
+      <c r="AR232"/>
     </row>
     <row r="233" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR233" s="32"/>
+      <c r="AR233"/>
     </row>
     <row r="234" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR234" s="32"/>
+      <c r="AR234"/>
     </row>
     <row r="235" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR235" s="32"/>
+      <c r="AR235"/>
     </row>
     <row r="236" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR236" s="32"/>
+      <c r="AR236"/>
     </row>
     <row r="237" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR237" s="32"/>
+      <c r="AR237"/>
     </row>
     <row r="238" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR238" s="32"/>
+      <c r="AR238"/>
     </row>
     <row r="239" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR239" s="32"/>
+      <c r="AR239"/>
     </row>
     <row r="240" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR240" s="32"/>
+      <c r="AR240"/>
     </row>
     <row r="241" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR241" s="32"/>
+      <c r="AR241"/>
     </row>
     <row r="242" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR242" s="32"/>
+      <c r="AR242"/>
     </row>
     <row r="243" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR243" s="32"/>
+      <c r="AR243"/>
     </row>
     <row r="244" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR244" s="32"/>
+      <c r="AR244"/>
     </row>
     <row r="245" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR245" s="32"/>
+      <c r="AR245"/>
     </row>
     <row r="246" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR246" s="32"/>
+      <c r="AR246"/>
     </row>
     <row r="247" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR247" s="32"/>
+      <c r="AR247"/>
     </row>
     <row r="248" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR248" s="32"/>
+      <c r="AR248"/>
     </row>
     <row r="249" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR249" s="32"/>
+      <c r="AR249"/>
     </row>
     <row r="250" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR250" s="32"/>
+      <c r="AR250"/>
     </row>
     <row r="251" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR251" s="32"/>
+      <c r="AR251"/>
     </row>
     <row r="252" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR252" s="32"/>
+      <c r="AR252"/>
     </row>
     <row r="253" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR253" s="32"/>
+      <c r="AR253"/>
     </row>
     <row r="254" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR254" s="32"/>
+      <c r="AR254"/>
     </row>
     <row r="255" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR255" s="32"/>
+      <c r="AR255"/>
     </row>
     <row r="256" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR256" s="32"/>
+      <c r="AR256"/>
     </row>
     <row r="257" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR257" s="32"/>
+      <c r="AR257"/>
     </row>
     <row r="258" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR258" s="32"/>
+      <c r="AR258"/>
     </row>
     <row r="259" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR259" s="32"/>
+      <c r="AR259"/>
     </row>
     <row r="260" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR260" s="32"/>
+      <c r="AR260"/>
     </row>
     <row r="261" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR261" s="32"/>
+      <c r="AR261"/>
     </row>
     <row r="262" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR262" s="32"/>
+      <c r="AR262"/>
     </row>
     <row r="263" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR263" s="32"/>
+      <c r="AR263"/>
     </row>
     <row r="264" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR264" s="32"/>
+      <c r="AR264"/>
     </row>
     <row r="265" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR265" s="32"/>
+      <c r="AR265"/>
     </row>
     <row r="266" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR266" s="32"/>
+      <c r="AR266"/>
     </row>
     <row r="267" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR267" s="32"/>
+      <c r="AR267"/>
     </row>
     <row r="268" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR268" s="32"/>
+      <c r="AR268"/>
     </row>
     <row r="269" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR269" s="32"/>
+      <c r="AR269"/>
     </row>
     <row r="270" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR270" s="32"/>
+      <c r="AR270"/>
     </row>
     <row r="271" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR271" s="32"/>
+      <c r="AR271"/>
     </row>
     <row r="272" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR272" s="32"/>
+      <c r="AR272"/>
     </row>
     <row r="273" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR273" s="32"/>
+      <c r="AR273"/>
     </row>
     <row r="274" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR274" s="32"/>
+      <c r="AR274"/>
     </row>
     <row r="275" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR275" s="32"/>
+      <c r="AR275"/>
     </row>
     <row r="276" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR276" s="32"/>
+      <c r="AR276"/>
     </row>
     <row r="277" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR277" s="32"/>
+      <c r="AR277"/>
     </row>
     <row r="278" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR278" s="32"/>
+      <c r="AR278"/>
     </row>
     <row r="279" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR279" s="32"/>
+      <c r="AR279"/>
     </row>
     <row r="280" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR280" s="32"/>
+      <c r="AR280"/>
     </row>
     <row r="281" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR281" s="32"/>
+      <c r="AR281"/>
     </row>
     <row r="282" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR282" s="32"/>
+      <c r="AR282"/>
     </row>
     <row r="283" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR283" s="32"/>
+      <c r="AR283"/>
     </row>
     <row r="284" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR284" s="32"/>
+      <c r="AR284"/>
     </row>
     <row r="285" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR285" s="32"/>
+      <c r="AR285"/>
     </row>
     <row r="286" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR286" s="32"/>
+      <c r="AR286"/>
     </row>
     <row r="287" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR287" s="32"/>
+      <c r="AR287"/>
     </row>
     <row r="288" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR288" s="32"/>
+      <c r="AR288"/>
     </row>
     <row r="289" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR289" s="32"/>
+      <c r="AR289"/>
     </row>
     <row r="290" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR290" s="32"/>
+      <c r="AR290"/>
     </row>
     <row r="291" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR291" s="32"/>
+      <c r="AR291"/>
     </row>
     <row r="292" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR292" s="32"/>
+      <c r="AR292"/>
     </row>
     <row r="293" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR293" s="32"/>
+      <c r="AR293"/>
     </row>
     <row r="294" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR294" s="32"/>
+      <c r="AR294"/>
     </row>
     <row r="295" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR295" s="32"/>
+      <c r="AR295"/>
     </row>
     <row r="296" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR296" s="32"/>
+      <c r="AR296"/>
     </row>
     <row r="297" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR297" s="32"/>
+      <c r="AR297"/>
     </row>
     <row r="298" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR298" s="32"/>
+      <c r="AR298"/>
     </row>
     <row r="299" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR299" s="32"/>
+      <c r="AR299"/>
     </row>
     <row r="300" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR300" s="32"/>
+      <c r="AR300"/>
     </row>
     <row r="301" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR301" s="32"/>
+      <c r="AR301"/>
     </row>
     <row r="302" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR302" s="32"/>
+      <c r="AR302"/>
     </row>
     <row r="303" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR303" s="32"/>
+      <c r="AR303"/>
     </row>
     <row r="304" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR304" s="32"/>
+      <c r="AR304"/>
     </row>
     <row r="305" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR305" s="32"/>
+      <c r="AR305"/>
     </row>
     <row r="306" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR306" s="32"/>
+      <c r="AR306"/>
     </row>
     <row r="307" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR307" s="32"/>
+      <c r="AR307"/>
     </row>
     <row r="308" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR308" s="32"/>
+      <c r="AR308"/>
     </row>
     <row r="309" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR309" s="32"/>
+      <c r="AR309"/>
     </row>
     <row r="310" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR310" s="32"/>
+      <c r="AR310"/>
     </row>
     <row r="311" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR311" s="32"/>
+      <c r="AR311"/>
     </row>
     <row r="312" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR312" s="32"/>
+      <c r="AR312"/>
     </row>
     <row r="313" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR313" s="32"/>
+      <c r="AR313"/>
     </row>
     <row r="314" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR314" s="32"/>
+      <c r="AR314"/>
     </row>
     <row r="315" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR315" s="32"/>
+      <c r="AR315"/>
     </row>
     <row r="316" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR316" s="32"/>
+      <c r="AR316"/>
     </row>
     <row r="317" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR317" s="32"/>
+      <c r="AR317"/>
     </row>
     <row r="318" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR318" s="32"/>
+      <c r="AR318"/>
     </row>
     <row r="319" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR319" s="32"/>
+      <c r="AR319"/>
     </row>
     <row r="320" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR320" s="32"/>
+      <c r="AR320"/>
     </row>
     <row r="321" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR321" s="32"/>
+      <c r="AR321"/>
     </row>
     <row r="322" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR322" s="32"/>
+      <c r="AR322"/>
     </row>
     <row r="323" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR323" s="32"/>
+      <c r="AR323"/>
     </row>
     <row r="324" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR324" s="32"/>
+      <c r="AR324"/>
     </row>
     <row r="325" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR325" s="32"/>
+      <c r="AR325"/>
     </row>
     <row r="326" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR326" s="32"/>
+      <c r="AR326"/>
     </row>
     <row r="327" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR327" s="32"/>
+      <c r="AR327"/>
     </row>
     <row r="328" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR328" s="32"/>
+      <c r="AR328"/>
     </row>
     <row r="329" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR329" s="32"/>
+      <c r="AR329"/>
     </row>
     <row r="330" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR330" s="32"/>
+      <c r="AR330"/>
     </row>
     <row r="331" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR331" s="32"/>
+      <c r="AR331"/>
     </row>
     <row r="332" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR332" s="32"/>
+      <c r="AR332"/>
     </row>
     <row r="333" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR333" s="32"/>
+      <c r="AR333"/>
     </row>
     <row r="334" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR334" s="32"/>
+      <c r="AR334"/>
     </row>
     <row r="335" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR335" s="32"/>
+      <c r="AR335"/>
     </row>
     <row r="336" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR336" s="32"/>
+      <c r="AR336"/>
     </row>
     <row r="337" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR337" s="32"/>
+      <c r="AR337"/>
     </row>
     <row r="338" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR338" s="32"/>
+      <c r="AR338"/>
     </row>
     <row r="339" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR339" s="32"/>
+      <c r="AR339"/>
     </row>
     <row r="340" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR340" s="32"/>
+      <c r="AR340"/>
     </row>
     <row r="341" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR341" s="32"/>
+      <c r="AR341"/>
     </row>
     <row r="342" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR342" s="32"/>
+      <c r="AR342"/>
     </row>
     <row r="343" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR343" s="32"/>
+      <c r="AR343"/>
     </row>
     <row r="344" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR344" s="32"/>
+      <c r="AR344"/>
     </row>
     <row r="345" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR345" s="32"/>
+      <c r="AR345"/>
     </row>
     <row r="346" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR346" s="32"/>
+      <c r="AR346"/>
     </row>
     <row r="347" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR347" s="32"/>
+      <c r="AR347"/>
     </row>
     <row r="348" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR348" s="32"/>
+      <c r="AR348"/>
     </row>
     <row r="349" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR349" s="32"/>
+      <c r="AR349"/>
     </row>
     <row r="350" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR350" s="32"/>
+      <c r="AR350"/>
     </row>
     <row r="351" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR351" s="32"/>
+      <c r="AR351"/>
     </row>
     <row r="352" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR352" s="32"/>
+      <c r="AR352"/>
     </row>
     <row r="353" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR353" s="32"/>
+      <c r="AR353"/>
     </row>
     <row r="354" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR354" s="32"/>
+      <c r="AR354"/>
     </row>
     <row r="355" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR355" s="32"/>
+      <c r="AR355"/>
     </row>
     <row r="356" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR356" s="32"/>
+      <c r="AR356"/>
     </row>
     <row r="357" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR357" s="32"/>
+      <c r="AR357"/>
     </row>
     <row r="358" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR358" s="32"/>
+      <c r="AR358"/>
     </row>
     <row r="359" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR359" s="32"/>
+      <c r="AR359"/>
     </row>
     <row r="360" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR360" s="32"/>
+      <c r="AR360"/>
     </row>
     <row r="361" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR361" s="32"/>
+      <c r="AR361"/>
     </row>
     <row r="362" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR362" s="32"/>
+      <c r="AR362"/>
     </row>
     <row r="363" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR363" s="32"/>
+      <c r="AR363"/>
     </row>
     <row r="364" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR364" s="32"/>
+      <c r="AR364"/>
     </row>
     <row r="365" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR365" s="32"/>
+      <c r="AR365"/>
     </row>
     <row r="366" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR366" s="32"/>
+      <c r="AR366"/>
     </row>
     <row r="367" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR367" s="32"/>
+      <c r="AR367"/>
     </row>
     <row r="368" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR368" s="32"/>
+      <c r="AR368"/>
     </row>
     <row r="369" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR369" s="32"/>
+      <c r="AR369"/>
     </row>
     <row r="370" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR370" s="32"/>
+      <c r="AR370"/>
     </row>
     <row r="371" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR371" s="32"/>
+      <c r="AR371"/>
     </row>
     <row r="372" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR372" s="32"/>
+      <c r="AR372"/>
     </row>
     <row r="373" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR373" s="32"/>
+      <c r="AR373"/>
     </row>
     <row r="374" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR374" s="32"/>
+      <c r="AR374"/>
     </row>
     <row r="375" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR375" s="32"/>
+      <c r="AR375"/>
     </row>
     <row r="376" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR376" s="32"/>
+      <c r="AR376"/>
     </row>
     <row r="377" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR377" s="32"/>
+      <c r="AR377"/>
     </row>
     <row r="378" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR378" s="32"/>
+      <c r="AR378"/>
     </row>
     <row r="379" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR379" s="32"/>
+      <c r="AR379"/>
     </row>
     <row r="380" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR380" s="32"/>
+      <c r="AR380"/>
     </row>
     <row r="381" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR381" s="32"/>
+      <c r="AR381"/>
     </row>
     <row r="382" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR382" s="32"/>
+      <c r="AR382"/>
     </row>
     <row r="383" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR383" s="32"/>
+      <c r="AR383"/>
     </row>
     <row r="384" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR384" s="32"/>
+      <c r="AR384"/>
     </row>
     <row r="385" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR385" s="32"/>
+      <c r="AR385"/>
     </row>
     <row r="386" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR386" s="32"/>
+      <c r="AR386"/>
     </row>
     <row r="387" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR387" s="32"/>
+      <c r="AR387"/>
     </row>
     <row r="388" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR388" s="32"/>
+      <c r="AR388"/>
     </row>
     <row r="389" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR389" s="32"/>
+      <c r="AR389"/>
     </row>
     <row r="390" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR390" s="32"/>
+      <c r="AR390"/>
     </row>
     <row r="391" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR391" s="32"/>
+      <c r="AR391"/>
     </row>
     <row r="392" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR392" s="32"/>
+      <c r="AR392"/>
     </row>
     <row r="393" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR393" s="32"/>
+      <c r="AR393"/>
     </row>
     <row r="394" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR394" s="32"/>
+      <c r="AR394"/>
     </row>
     <row r="395" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR395" s="32"/>
+      <c r="AR395"/>
     </row>
     <row r="396" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR396" s="32"/>
+      <c r="AR396"/>
     </row>
     <row r="397" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR397" s="32"/>
+      <c r="AR397"/>
     </row>
     <row r="398" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR398" s="32"/>
+      <c r="AR398"/>
     </row>
     <row r="399" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR399" s="32"/>
+      <c r="AR399"/>
     </row>
     <row r="400" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR400" s="32"/>
+      <c r="AR400"/>
     </row>
     <row r="401" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR401" s="32"/>
+      <c r="AR401"/>
     </row>
     <row r="402" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR402" s="32"/>
+      <c r="AR402"/>
     </row>
     <row r="403" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR403" s="32"/>
+      <c r="AR403"/>
     </row>
     <row r="404" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR404" s="32"/>
+      <c r="AR404"/>
     </row>
     <row r="405" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR405" s="32"/>
+      <c r="AR405"/>
     </row>
     <row r="406" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR406" s="32"/>
+      <c r="AR406"/>
     </row>
     <row r="407" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR407" s="32"/>
+      <c r="AR407"/>
     </row>
     <row r="408" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR408" s="32"/>
+      <c r="AR408"/>
     </row>
     <row r="409" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR409" s="32"/>
+      <c r="AR409"/>
     </row>
     <row r="410" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR410" s="32"/>
+      <c r="AR410"/>
     </row>
     <row r="411" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR411" s="32"/>
+      <c r="AR411"/>
     </row>
     <row r="412" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR412" s="32"/>
+      <c r="AR412"/>
     </row>
     <row r="413" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR413" s="32"/>
+      <c r="AR413"/>
     </row>
     <row r="414" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR414" s="32"/>
+      <c r="AR414"/>
     </row>
     <row r="415" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR415" s="32"/>
+      <c r="AR415"/>
     </row>
     <row r="416" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR416" s="32"/>
+      <c r="AR416"/>
     </row>
     <row r="417" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR417" s="32"/>
+      <c r="AR417"/>
     </row>
     <row r="418" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR418" s="32"/>
+      <c r="AR418"/>
     </row>
     <row r="419" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR419" s="32"/>
+      <c r="AR419"/>
     </row>
     <row r="420" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR420" s="32"/>
+      <c r="AR420"/>
     </row>
     <row r="421" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR421" s="32"/>
+      <c r="AR421"/>
     </row>
     <row r="422" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR422" s="32"/>
+      <c r="AR422"/>
     </row>
     <row r="423" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR423" s="32"/>
+      <c r="AR423"/>
     </row>
     <row r="424" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR424" s="32"/>
+      <c r="AR424"/>
     </row>
     <row r="425" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR425" s="32"/>
+      <c r="AR425"/>
     </row>
     <row r="426" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR426" s="32"/>
+      <c r="AR426"/>
     </row>
     <row r="427" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR427" s="32"/>
+      <c r="AR427"/>
     </row>
     <row r="428" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR428" s="32"/>
+      <c r="AR428"/>
     </row>
     <row r="429" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR429" s="32"/>
+      <c r="AR429"/>
     </row>
     <row r="430" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR430" s="32"/>
+      <c r="AR430"/>
     </row>
     <row r="431" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR431" s="32"/>
+      <c r="AR431"/>
     </row>
     <row r="432" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR432" s="32"/>
+      <c r="AR432"/>
     </row>
     <row r="433" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR433" s="32"/>
+      <c r="AR433"/>
     </row>
     <row r="434" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR434" s="32"/>
+      <c r="AR434"/>
     </row>
     <row r="435" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR435" s="32"/>
+      <c r="AR435"/>
     </row>
     <row r="436" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR436" s="32"/>
+      <c r="AR436"/>
     </row>
     <row r="437" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR437" s="32"/>
+      <c r="AR437"/>
     </row>
     <row r="438" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR438" s="32"/>
+      <c r="AR438"/>
     </row>
     <row r="439" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR439" s="32"/>
+      <c r="AR439"/>
     </row>
     <row r="440" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR440" s="32"/>
+      <c r="AR440"/>
     </row>
     <row r="441" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR441" s="32"/>
+      <c r="AR441"/>
     </row>
     <row r="442" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR442" s="32"/>
+      <c r="AR442"/>
     </row>
     <row r="443" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR443" s="32"/>
+      <c r="AR443"/>
     </row>
     <row r="444" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR444" s="32"/>
+      <c r="AR444"/>
     </row>
     <row r="445" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR445" s="32"/>
+      <c r="AR445"/>
     </row>
     <row r="446" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR446" s="32"/>
+      <c r="AR446"/>
     </row>
     <row r="447" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR447" s="32"/>
+      <c r="AR447"/>
     </row>
     <row r="448" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR448" s="32"/>
+      <c r="AR448"/>
     </row>
     <row r="449" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR449" s="32"/>
+      <c r="AR449"/>
     </row>
     <row r="450" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR450" s="32"/>
+      <c r="AR450"/>
     </row>
     <row r="451" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR451" s="32"/>
+      <c r="AR451"/>
     </row>
     <row r="452" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR452" s="32"/>
+      <c r="AR452"/>
     </row>
     <row r="453" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR453" s="32"/>
+      <c r="AR453"/>
     </row>
     <row r="454" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR454" s="32"/>
+      <c r="AR454"/>
     </row>
     <row r="455" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR455" s="32"/>
+      <c r="AR455"/>
     </row>
     <row r="456" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR456" s="32"/>
+      <c r="AR456"/>
     </row>
     <row r="457" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR457" s="32"/>
+      <c r="AR457"/>
     </row>
     <row r="458" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR458" s="32"/>
+      <c r="AR458"/>
     </row>
     <row r="459" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR459" s="32"/>
+      <c r="AR459"/>
     </row>
     <row r="460" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR460" s="32"/>
+      <c r="AR460"/>
     </row>
     <row r="461" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR461" s="32"/>
+      <c r="AR461"/>
     </row>
     <row r="462" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR462" s="32"/>
+      <c r="AR462"/>
     </row>
     <row r="463" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR463" s="32"/>
+      <c r="AR463"/>
     </row>
     <row r="464" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR464" s="32"/>
+      <c r="AR464"/>
     </row>
     <row r="465" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR465" s="32"/>
+      <c r="AR465"/>
     </row>
     <row r="466" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR466" s="32"/>
+      <c r="AR466"/>
     </row>
     <row r="467" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR467" s="32"/>
+      <c r="AR467"/>
     </row>
     <row r="468" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR468" s="32"/>
+      <c r="AR468"/>
     </row>
     <row r="469" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR469" s="32"/>
+      <c r="AR469"/>
     </row>
     <row r="470" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR470" s="32"/>
+      <c r="AR470"/>
     </row>
     <row r="471" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR471" s="32"/>
+      <c r="AR471"/>
     </row>
     <row r="472" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR472" s="32"/>
+      <c r="AR472"/>
     </row>
     <row r="473" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR473" s="32"/>
+      <c r="AR473"/>
     </row>
     <row r="474" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR474" s="32"/>
+      <c r="AR474"/>
     </row>
     <row r="475" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR475" s="32"/>
+      <c r="AR475"/>
     </row>
     <row r="476" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR476" s="32"/>
+      <c r="AR476"/>
     </row>
     <row r="477" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR477" s="32"/>
+      <c r="AR477"/>
     </row>
     <row r="478" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR478" s="32"/>
+      <c r="AR478"/>
     </row>
     <row r="479" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR479" s="32"/>
+      <c r="AR479"/>
     </row>
     <row r="480" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR480" s="32"/>
+      <c r="AR480"/>
     </row>
     <row r="481" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR481" s="32"/>
+      <c r="AR481"/>
     </row>
     <row r="482" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR482" s="32"/>
+      <c r="AR482"/>
     </row>
     <row r="483" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR483" s="32"/>
+      <c r="AR483"/>
     </row>
     <row r="484" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR484" s="32"/>
+      <c r="AR484"/>
     </row>
     <row r="485" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR485" s="32"/>
+      <c r="AR485"/>
     </row>
     <row r="486" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR486" s="32"/>
+      <c r="AR486"/>
     </row>
     <row r="487" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR487" s="32"/>
+      <c r="AR487"/>
     </row>
     <row r="488" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR488" s="32"/>
+      <c r="AR488"/>
     </row>
     <row r="489" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR489" s="32"/>
+      <c r="AR489"/>
     </row>
     <row r="490" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR490" s="32"/>
+      <c r="AR490"/>
     </row>
     <row r="491" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR491" s="32"/>
+      <c r="AR491"/>
     </row>
     <row r="492" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR492" s="32"/>
+      <c r="AR492"/>
     </row>
     <row r="493" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR493" s="32"/>
+      <c r="AR493"/>
     </row>
     <row r="494" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR494" s="32"/>
+      <c r="AR494"/>
     </row>
     <row r="495" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR495" s="32"/>
+      <c r="AR495"/>
     </row>
     <row r="496" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR496" s="32"/>
+      <c r="AR496"/>
     </row>
     <row r="497" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR497" s="32"/>
+      <c r="AR497"/>
     </row>
     <row r="498" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR498" s="32"/>
+      <c r="AR498"/>
     </row>
     <row r="499" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR499" s="32"/>
+      <c r="AR499"/>
     </row>
     <row r="500" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR500" s="32"/>
+      <c r="AR500"/>
     </row>
     <row r="501" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR501" s="32"/>
+      <c r="AR501"/>
     </row>
     <row r="502" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR502" s="32"/>
+      <c r="AR502"/>
     </row>
     <row r="503" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR503" s="32"/>
+      <c r="AR503"/>
     </row>
     <row r="504" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR504" s="32"/>
+      <c r="AR504"/>
     </row>
     <row r="505" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR505" s="32"/>
+      <c r="AR505"/>
     </row>
     <row r="506" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR506" s="32"/>
+      <c r="AR506"/>
     </row>
     <row r="507" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR507" s="32"/>
+      <c r="AR507"/>
     </row>
     <row r="508" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR508" s="32"/>
+      <c r="AR508"/>
     </row>
     <row r="509" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR509" s="32"/>
+      <c r="AR509"/>
     </row>
     <row r="510" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR510" s="32"/>
+      <c r="AR510"/>
     </row>
     <row r="511" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR511" s="32"/>
+      <c r="AR511"/>
     </row>
     <row r="512" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR512" s="32"/>
+      <c r="AR512"/>
     </row>
     <row r="513" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR513" s="32"/>
+      <c r="AR513"/>
     </row>
     <row r="514" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR514" s="32"/>
+      <c r="AR514"/>
     </row>
     <row r="515" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR515" s="32"/>
+      <c r="AR515"/>
     </row>
     <row r="516" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR516" s="32"/>
+      <c r="AR516"/>
     </row>
     <row r="517" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR517" s="32"/>
+      <c r="AR517"/>
     </row>
     <row r="518" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR518" s="32"/>
+      <c r="AR518"/>
     </row>
     <row r="519" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR519" s="32"/>
+      <c r="AR519"/>
     </row>
     <row r="520" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR520" s="32"/>
+      <c r="AR520"/>
     </row>
     <row r="521" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR521" s="32"/>
+      <c r="AR521"/>
     </row>
     <row r="522" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR522" s="32"/>
+      <c r="AR522"/>
     </row>
     <row r="523" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR523" s="32"/>
+      <c r="AR523"/>
     </row>
     <row r="524" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR524" s="32"/>
+      <c r="AR524"/>
     </row>
     <row r="525" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR525" s="32"/>
+      <c r="AR525"/>
     </row>
     <row r="526" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR526" s="32"/>
+      <c r="AR526"/>
     </row>
     <row r="527" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR527" s="32"/>
+      <c r="AR527"/>
     </row>
     <row r="528" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR528" s="32"/>
+      <c r="AR528"/>
     </row>
     <row r="529" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR529" s="32"/>
+      <c r="AR529"/>
     </row>
     <row r="530" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR530" s="32"/>
+      <c r="AR530"/>
     </row>
     <row r="531" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR531" s="32"/>
+      <c r="AR531"/>
     </row>
     <row r="532" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR532" s="32"/>
+      <c r="AR532"/>
     </row>
     <row r="533" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR533" s="32"/>
+      <c r="AR533"/>
     </row>
     <row r="534" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR534" s="32"/>
+      <c r="AR534"/>
     </row>
     <row r="535" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR535" s="32"/>
+      <c r="AR535"/>
     </row>
     <row r="536" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR536" s="32"/>
+      <c r="AR536"/>
     </row>
     <row r="537" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR537" s="32"/>
+      <c r="AR537"/>
     </row>
     <row r="538" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR538" s="32"/>
+      <c r="AR538"/>
     </row>
     <row r="539" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR539" s="32"/>
+      <c r="AR539"/>
     </row>
     <row r="540" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR540" s="32"/>
+      <c r="AR540"/>
     </row>
     <row r="541" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR541" s="32"/>
+      <c r="AR541"/>
     </row>
     <row r="542" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR542" s="32"/>
+      <c r="AR542"/>
     </row>
     <row r="543" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR543" s="32"/>
+      <c r="AR543"/>
     </row>
     <row r="544" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR544" s="32"/>
+      <c r="AR544"/>
     </row>
     <row r="545" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR545" s="32"/>
+      <c r="AR545"/>
     </row>
     <row r="546" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR546" s="32"/>
+      <c r="AR546"/>
     </row>
     <row r="547" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR547" s="32"/>
+      <c r="AR547"/>
     </row>
     <row r="548" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR548" s="32"/>
+      <c r="AR548"/>
     </row>
     <row r="549" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR549" s="32"/>
+      <c r="AR549"/>
     </row>
     <row r="550" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR550" s="32"/>
+      <c r="AR550"/>
     </row>
     <row r="551" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR551" s="32"/>
+      <c r="AR551"/>
     </row>
     <row r="552" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR552" s="32"/>
+      <c r="AR552"/>
     </row>
     <row r="553" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR553" s="32"/>
+      <c r="AR553"/>
     </row>
     <row r="554" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR554" s="32"/>
+      <c r="AR554"/>
     </row>
     <row r="555" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR555" s="32"/>
+      <c r="AR555"/>
     </row>
     <row r="556" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR556" s="32"/>
+      <c r="AR556"/>
     </row>
     <row r="557" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR557" s="32"/>
+      <c r="AR557"/>
     </row>
     <row r="558" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR558" s="32"/>
+      <c r="AR558"/>
     </row>
     <row r="559" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR559" s="32"/>
+      <c r="AR559"/>
     </row>
     <row r="560" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR560" s="32"/>
+      <c r="AR560"/>
     </row>
     <row r="561" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR561" s="32"/>
+      <c r="AR561"/>
     </row>
     <row r="562" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR562" s="32"/>
+      <c r="AR562"/>
     </row>
     <row r="563" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR563" s="32"/>
+      <c r="AR563"/>
     </row>
     <row r="564" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR564" s="32"/>
+      <c r="AR564"/>
     </row>
     <row r="565" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR565" s="32"/>
+      <c r="AR565"/>
     </row>
     <row r="566" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR566" s="32"/>
+      <c r="AR566"/>
     </row>
     <row r="567" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR567" s="32"/>
+      <c r="AR567"/>
     </row>
     <row r="568" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR568" s="32"/>
+      <c r="AR568"/>
     </row>
     <row r="569" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR569" s="32"/>
+      <c r="AR569"/>
     </row>
     <row r="570" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR570" s="32"/>
+      <c r="AR570"/>
     </row>
     <row r="571" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR571" s="32"/>
+      <c r="AR571"/>
     </row>
     <row r="572" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR572" s="32"/>
+      <c r="AR572"/>
     </row>
     <row r="573" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR573" s="32"/>
+      <c r="AR573"/>
     </row>
     <row r="574" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR574" s="32"/>
+      <c r="AR574"/>
     </row>
     <row r="575" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR575" s="32"/>
+      <c r="AR575"/>
     </row>
     <row r="576" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR576" s="32"/>
+      <c r="AR576"/>
     </row>
     <row r="577" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR577" s="32"/>
+      <c r="AR577"/>
     </row>
     <row r="578" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR578" s="32"/>
+      <c r="AR578"/>
     </row>
     <row r="579" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR579" s="32"/>
+      <c r="AR579"/>
     </row>
     <row r="580" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR580" s="32"/>
+      <c r="AR580"/>
     </row>
     <row r="581" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR581" s="32"/>
+      <c r="AR581"/>
     </row>
     <row r="582" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR582" s="32"/>
+      <c r="AR582"/>
     </row>
     <row r="583" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR583" s="32"/>
+      <c r="AR583"/>
     </row>
     <row r="584" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR584" s="32"/>
+      <c r="AR584"/>
     </row>
     <row r="585" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR585" s="32"/>
+      <c r="AR585"/>
     </row>
     <row r="586" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR586" s="32"/>
+      <c r="AR586"/>
     </row>
     <row r="587" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR587" s="32"/>
+      <c r="AR587"/>
     </row>
     <row r="588" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR588" s="32"/>
+      <c r="AR588"/>
     </row>
     <row r="589" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR589" s="32"/>
+      <c r="AR589"/>
     </row>
     <row r="590" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR590" s="32"/>
+      <c r="AR590"/>
     </row>
     <row r="591" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR591" s="32"/>
+      <c r="AR591"/>
     </row>
     <row r="592" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR592" s="32"/>
+      <c r="AR592"/>
     </row>
     <row r="593" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR593" s="32"/>
+      <c r="AR593"/>
     </row>
     <row r="594" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR594" s="32"/>
+      <c r="AR594"/>
     </row>
     <row r="595" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR595" s="32"/>
+      <c r="AR595"/>
     </row>
     <row r="596" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR596" s="32"/>
+      <c r="AR596"/>
     </row>
     <row r="597" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR597" s="32"/>
+      <c r="AR597"/>
     </row>
     <row r="598" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR598" s="32"/>
+      <c r="AR598"/>
     </row>
     <row r="599" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR599" s="32"/>
+      <c r="AR599"/>
     </row>
     <row r="600" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR600" s="32"/>
+      <c r="AR600"/>
     </row>
     <row r="601" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR601" s="32"/>
+      <c r="AR601"/>
     </row>
     <row r="602" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR602" s="32"/>
+      <c r="AR602"/>
     </row>
     <row r="603" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR603" s="32"/>
+      <c r="AR603"/>
     </row>
     <row r="604" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR604" s="32"/>
+      <c r="AR604"/>
     </row>
     <row r="605" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR605" s="32"/>
+      <c r="AR605"/>
     </row>
     <row r="606" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR606" s="32"/>
+      <c r="AR606"/>
     </row>
     <row r="607" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR607" s="32"/>
+      <c r="AR607"/>
     </row>
     <row r="608" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR608" s="32"/>
+      <c r="AR608"/>
     </row>
     <row r="609" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR609" s="32"/>
+      <c r="AR609"/>
     </row>
     <row r="610" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR610" s="32"/>
+      <c r="AR610"/>
     </row>
     <row r="611" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR611" s="32"/>
+      <c r="AR611"/>
     </row>
     <row r="612" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR612" s="32"/>
+      <c r="AR612"/>
     </row>
     <row r="613" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR613" s="32"/>
+      <c r="AR613"/>
     </row>
     <row r="614" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR614" s="32"/>
+      <c r="AR614"/>
     </row>
     <row r="615" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR615" s="32"/>
+      <c r="AR615"/>
     </row>
     <row r="616" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR616" s="32"/>
+      <c r="AR616"/>
     </row>
     <row r="617" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR617" s="32"/>
+      <c r="AR617"/>
     </row>
     <row r="618" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR618" s="32"/>
+      <c r="AR618"/>
     </row>
     <row r="619" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR619" s="32"/>
+      <c r="AR619"/>
     </row>
     <row r="620" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR620" s="32"/>
+      <c r="AR620"/>
     </row>
     <row r="621" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR621" s="32"/>
+      <c r="AR621"/>
     </row>
     <row r="622" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR622" s="32"/>
+      <c r="AR622"/>
     </row>
     <row r="623" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR623" s="32"/>
+      <c r="AR623"/>
     </row>
     <row r="624" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR624" s="32"/>
+      <c r="AR624"/>
     </row>
     <row r="625" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR625" s="32"/>
+      <c r="AR625"/>
     </row>
     <row r="626" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR626" s="32"/>
+      <c r="AR626"/>
     </row>
     <row r="627" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR627" s="32"/>
+      <c r="AR627"/>
     </row>
     <row r="628" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR628" s="32"/>
+      <c r="AR628"/>
     </row>
     <row r="629" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR629" s="32"/>
+      <c r="AR629"/>
     </row>
     <row r="630" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR630" s="32"/>
+      <c r="AR630"/>
     </row>
     <row r="631" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR631" s="32"/>
+      <c r="AR631"/>
     </row>
     <row r="632" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR632" s="32"/>
+      <c r="AR632"/>
     </row>
     <row r="633" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR633" s="32"/>
+      <c r="AR633"/>
     </row>
     <row r="634" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR634" s="32"/>
+      <c r="AR634"/>
     </row>
     <row r="635" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR635" s="32"/>
+      <c r="AR635"/>
     </row>
     <row r="636" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR636" s="32"/>
+      <c r="AR636"/>
     </row>
     <row r="637" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR637" s="32"/>
+      <c r="AR637"/>
     </row>
     <row r="638" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR638" s="32"/>
+      <c r="AR638"/>
     </row>
     <row r="639" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR639" s="32"/>
+      <c r="AR639"/>
     </row>
     <row r="640" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR640" s="32"/>
+      <c r="AR640"/>
     </row>
     <row r="641" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR641" s="32"/>
+      <c r="AR641"/>
     </row>
     <row r="642" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR642" s="32"/>
+      <c r="AR642"/>
     </row>
     <row r="643" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR643" s="32"/>
+      <c r="AR643"/>
     </row>
     <row r="644" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR644" s="32"/>
+      <c r="AR644"/>
     </row>
     <row r="645" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR645" s="32"/>
+      <c r="AR645"/>
     </row>
     <row r="646" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR646" s="32"/>
+      <c r="AR646"/>
     </row>
     <row r="647" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR647" s="32"/>
+      <c r="AR647"/>
     </row>
     <row r="648" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR648" s="32"/>
+      <c r="AR648"/>
     </row>
     <row r="649" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR649" s="32"/>
+      <c r="AR649"/>
     </row>
     <row r="650" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR650" s="32"/>
+      <c r="AR650"/>
     </row>
     <row r="651" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR651" s="32"/>
+      <c r="AR651"/>
     </row>
     <row r="652" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR652" s="32"/>
+      <c r="AR652"/>
     </row>
     <row r="653" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR653" s="32"/>
+      <c r="AR653"/>
     </row>
     <row r="654" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR654" s="32"/>
+      <c r="AR654"/>
     </row>
     <row r="655" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR655" s="32"/>
+      <c r="AR655"/>
     </row>
     <row r="656" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR656" s="32"/>
+      <c r="AR656"/>
     </row>
     <row r="657" spans="44:44" x14ac:dyDescent="0.3">
-      <c r="AR657" s="32"/>
+      <c r="AR657"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>